<commit_message>
feat: batch 1 des illustrations SET01 — 12 remplacements, 5 nouvelles cartes, 5 arts alternatifs
- Forge --replace : R01-R10, R13 (transfert-durgence), R16 (viktor-volkov)
- Nouvelles cartes : porteur-de-cell-vole (K05), senior-descorte (R12),
  bouclier-de-plateforme (R14), porteur-cell-magnus (R17), allocation-denergie (R18)
- Doublons du drop stockés en arts alternatifs (static/art/alt/)
- Tableau de production régénéré (xlsx + csv) — 23/60 forgées

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/SET01-production.xlsx
+++ b/docs/SET01-production.xlsx
@@ -1528,9 +1528,9 @@
           <t>senior-descorte</t>
         </is>
       </c>
-      <c r="C13" s="6" t="inlineStr">
-        <is>
-          <t>À générer</t>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Forgée</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
@@ -1551,13 +1551,29 @@
       <c r="G13" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="H13" s="2" t="inlineStr"/>
-      <c r="I13" s="2" t="inlineStr"/>
-      <c r="J13" s="2" t="inlineStr"/>
-      <c r="K13" s="5" t="inlineStr"/>
+      <c r="H13" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I13" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>CELL de série · Bastion</t>
+        </is>
+      </c>
+      <c r="K13" s="5" t="inlineStr">
+        <is>
+          <t>Garde.</t>
+        </is>
+      </c>
       <c r="L13" s="2" t="inlineStr"/>
       <c r="M13" s="5" t="inlineStr"/>
-      <c r="N13" s="5" t="inlineStr"/>
+      <c r="N13" s="5" t="inlineStr">
+        <is>
+          <t>Trois cycles de recrues lui ont survécu. C'est le but.</t>
+        </is>
+      </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
           <t>Non</t>
@@ -1670,9 +1686,9 @@
           <t>bouclier-de-plateforme</t>
         </is>
       </c>
-      <c r="C15" s="6" t="inlineStr">
-        <is>
-          <t>À générer</t>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>Forgée</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
@@ -1696,10 +1712,18 @@
       <c r="H15" s="2" t="inlineStr"/>
       <c r="I15" s="2" t="inlineStr"/>
       <c r="J15" s="2" t="inlineStr"/>
-      <c r="K15" s="5" t="inlineStr"/>
+      <c r="K15" s="5" t="inlineStr">
+        <is>
+          <t>Vos unités gagnent +0/+2.</t>
+        </is>
+      </c>
       <c r="L15" s="2" t="inlineStr"/>
       <c r="M15" s="5" t="inlineStr"/>
-      <c r="N15" s="5" t="inlineStr"/>
+      <c r="N15" s="5" t="inlineStr">
+        <is>
+          <t>Le dôme tient tant que la Centrale respire.</t>
+        </is>
+      </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
           <t>Non</t>
@@ -1893,9 +1917,9 @@
           <t>porteur-cell-magnus</t>
         </is>
       </c>
-      <c r="C18" s="6" t="inlineStr">
-        <is>
-          <t>À générer</t>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>Forgée</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
@@ -1916,13 +1940,31 @@
       <c r="G18" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="H18" s="2" t="inlineStr"/>
-      <c r="I18" s="2" t="inlineStr"/>
-      <c r="J18" s="2" t="inlineStr"/>
+      <c r="H18" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="I18" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>CELL Magnus</t>
+        </is>
+      </c>
       <c r="K18" s="5" t="inlineStr"/>
-      <c r="L18" s="2" t="inlineStr"/>
-      <c r="M18" s="5" t="inlineStr"/>
-      <c r="N18" s="5" t="inlineStr"/>
+      <c r="L18" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="M18" s="5" t="inlineStr">
+        <is>
+          <t>Magnétosphère : vos autres Travelers gagnent +1/+1.</t>
+        </is>
+      </c>
+      <c r="N18" s="5" t="inlineStr">
+        <is>
+          <t>Le fer se souvient de lui.</t>
+        </is>
+      </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
           <t>Non</t>
@@ -1960,9 +2002,9 @@
           <t>allocation-denergie</t>
         </is>
       </c>
-      <c r="C19" s="6" t="inlineStr">
-        <is>
-          <t>À générer</t>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>Forgée</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
@@ -1986,10 +2028,18 @@
       <c r="H19" s="2" t="inlineStr"/>
       <c r="I19" s="2" t="inlineStr"/>
       <c r="J19" s="2" t="inlineStr"/>
-      <c r="K19" s="5" t="inlineStr"/>
+      <c r="K19" s="5" t="inlineStr">
+        <is>
+          <t>Ce tour-ci, vos Synchros coûtent (0).</t>
+        </is>
+      </c>
       <c r="L19" s="2" t="inlineStr"/>
       <c r="M19" s="5" t="inlineStr"/>
-      <c r="N19" s="5" t="inlineStr"/>
+      <c r="N19" s="5" t="inlineStr">
+        <is>
+          <t>La Centrale a hurlé six secondes. Toutes les équipes s'en souviennent.</t>
+        </is>
+      </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
           <t>Non</t>
@@ -2623,9 +2673,9 @@
           <t>porteur-de-cell-vole</t>
         </is>
       </c>
-      <c r="C28" s="6" t="inlineStr">
-        <is>
-          <t>À générer</t>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>Forgée</t>
         </is>
       </c>
       <c r="D28" s="7" t="inlineStr">
@@ -2646,13 +2696,29 @@
       <c r="G28" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H28" s="2" t="inlineStr"/>
-      <c r="I28" s="2" t="inlineStr"/>
-      <c r="J28" s="2" t="inlineStr"/>
-      <c r="K28" s="5" t="inlineStr"/>
+      <c r="H28" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I28" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>CELL volé · sans registre</t>
+        </is>
+      </c>
+      <c r="K28" s="5" t="inlineStr">
+        <is>
+          <t>Célérité.</t>
+        </is>
+      </c>
       <c r="L28" s="2" t="inlineStr"/>
       <c r="M28" s="5" t="inlineStr"/>
-      <c r="N28" s="5" t="inlineStr"/>
+      <c r="N28" s="5" t="inlineStr">
+        <is>
+          <t>Le suit grésille. Il s'en fout.</t>
+        </is>
+      </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
           <t>Non</t>

</xml_diff>

<commit_message>
docs: prompts MJ sans style peinture ni --ar (réglés par défaut côté Midjourney) ; tableau régénéré
- PROMPTS.md : suppression de 'dark epic digital painting', 'painterly
  brushstrokes', 'painterly' et de tous les '--ar 4:5' (60 prompts) ;
  métaphores picturales des slots E13/E16 reformulées ; note d'entête à jour
- charter.json : basePrompt allégé des termes peinture
- SET01-production.xlsx + csv régénérés

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/SET01-production.xlsx
+++ b/docs/SET01-production.xlsx
@@ -709,7 +709,7 @@
       </c>
       <c r="S2" s="5" t="inlineStr">
         <is>
-          <t>young female recruit in a plain matte black pre-CELL training bodysuit with small sensor pads, standing alert in a dark underground RIKKEN training hall, black metal walls with faint blue LED strips, determined tired eyes, subject centered upper half, dark epic digital painting, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated blue accent #3d8fd6, painterly brushstrokes, seinen atmosphere --ar 4:5 --no neon everywhere, rainbow colors, iron man style, text, watermark</t>
+          <t>young female recruit in a plain matte black pre-CELL training bodysuit with small sensor pads, standing alert in a dark underground RIKKEN training hall, black metal walls with faint blue LED strips, determined tired eyes, subject centered upper half, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated blue accent #3d8fd6, seinen atmosphere --no neon everywhere, rainbow colors, iron man style, text, watermark</t>
         </is>
       </c>
     </row>
@@ -792,7 +792,7 @@
       </c>
       <c r="S3" s="5" t="inlineStr">
         <is>
-          <t>female engineer in dark RIKKEN work uniform and cap repairing massive energy conduits deep under Odaiba, cold blue-white glow of the transfer core lighting her face from below, wrench in hand, cathedral-scale machinery, subject centered upper half, dark epic digital painting, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated blue accent #3d8fd6, painterly brushstrokes, seinen atmosphere --ar 4:5 --no neon everywhere, rainbow colors, text, watermark</t>
+          <t>female engineer in dark RIKKEN work uniform and cap repairing massive energy conduits deep under Odaiba, cold blue-white glow of the transfer core lighting her face from below, wrench in hand, cathedral-scale machinery, subject centered upper half, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated blue accent #3d8fd6, seinen atmosphere --no neon everywhere, rainbow colors, text, watermark</t>
         </is>
       </c>
     </row>
@@ -877,7 +877,7 @@
       </c>
       <c r="S4" s="5" t="inlineStr">
         <is>
-          <t>female operative in a sleek black biotech suit with modular plates, thin water conduits glowing soft cyan along forearms and collar, fine mist condensing around her hands, calm ready stance in a dark concrete hall, subject centered upper half, dark epic digital painting, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated cyan accent, contained light lines, painterly, seinen atmosphere --ar 4:5 --no neon everywhere, rainbow colors, iron man style, text, watermark</t>
+          <t>female operative in a sleek black biotech suit with modular plates, thin water conduits glowing soft cyan along forearms and collar, fine mist condensing around her hands, calm ready stance in a dark concrete hall, subject centered upper half, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated cyan accent, contained light lines, seinen atmosphere --no neon everywhere, rainbow colors, iron man style, text, watermark</t>
         </is>
       </c>
     </row>
@@ -960,7 +960,7 @@
       </c>
       <c r="S5" s="5" t="inlineStr">
         <is>
-          <t>female scout in a sleek dark biotech suit sprinting through a foggy 19th century parisian construction site at night, wooden scaffolding and iron beams in the mist, subtle motion blur, aerodynamic suit panels with faint blue light lines, subject centered upper half, dark epic digital painting, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated blue accent #3d8fd6, painterly brushstrokes, seinen atmosphere --ar 4:5 --no neon everywhere, rainbow colors, eiffel tower recognizable, text, watermark</t>
+          <t>female scout in a sleek dark biotech suit sprinting through a foggy 19th century parisian construction site at night, wooden scaffolding and iron beams in the mist, subtle motion blur, aerodynamic suit panels with faint blue light lines, subject centered upper half, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated blue accent #3d8fd6, seinen atmosphere --no neon everywhere, rainbow colors, eiffel tower recognizable, text, watermark</t>
         </is>
       </c>
     </row>
@@ -1043,7 +1043,7 @@
       </c>
       <c r="S6" s="5" t="inlineStr">
         <is>
-          <t>massive sentinel in a heavy-plated dark biotech suit standing guard before a circular time-transfer platform, faint blue-white glow rising from the platform ring behind him, arms crossed, immovable, black metal hall with blue LED strips, subject centered upper half, dark epic digital painting, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated blue accent #3d8fd6, painterly, seinen atmosphere --ar 4:5 --no neon everywhere, rainbow colors, iron man style, giant mecha, text, watermark</t>
+          <t>massive sentinel in a heavy-plated dark biotech suit standing guard before a circular time-transfer platform, faint blue-white glow rising from the platform ring behind him, arms crossed, immovable, black metal hall with blue LED strips, subject centered upper half, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated blue accent #3d8fd6, seinen atmosphere --no neon everywhere, rainbow colors, iron man style, giant mecha, text, watermark</t>
         </is>
       </c>
     </row>
@@ -1126,7 +1126,7 @@
       </c>
       <c r="S7" s="5" t="inlineStr">
         <is>
-          <t>stern analyst in dark institutional uniform at a desk of translucent holographic timelines and candidate files, glasses reflecting pale blue data, dark office of the recruitment division at night, subject centered upper half, dark epic digital painting, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated blue accent #3d8fd6, painterly brushstrokes, seinen atmosphere --ar 4:5 --no neon everywhere, rainbow colors, cyberpunk pink purple, text, watermark</t>
+          <t>stern analyst in dark institutional uniform at a desk of translucent holographic timelines and candidate files, glasses reflecting pale blue data, dark office of the recruitment division at night, subject centered upper half, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated blue accent #3d8fd6, seinen atmosphere --no neon everywhere, rainbow colors, cyberpunk pink purple, text, watermark</t>
         </is>
       </c>
     </row>
@@ -1201,7 +1201,7 @@
       </c>
       <c r="S8" s="5" t="inlineStr">
         <is>
-          <t>human silhouette dissolving into fine ascending blue-white light lines on a circular transfer platform, empty dark facility, the light column is the only bright source, sense of sudden departure, a dropped object still falling where the person stood, dark epic digital painting, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated blue accent #3d8fd6, painterly, seinen atmosphere --ar 4:5 --no neon everywhere, rainbow colors, text, watermark</t>
+          <t>human silhouette dissolving into fine ascending blue-white light lines on a circular transfer platform, empty dark facility, the light column is the only bright source, sense of sudden departure, a dropped object still falling where the person stood, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated blue accent #3d8fd6, seinen atmosphere --no neon everywhere, rainbow colors, text, watermark</t>
         </is>
       </c>
     </row>
@@ -1276,7 +1276,7 @@
       </c>
       <c r="S9" s="5" t="inlineStr">
         <is>
-          <t>holographic briefing table projecting layered maps of seven different historical eras, gloved hands of unseen officers pointing at a blank unmapped region, dark war-room of the RIKKEN facility, papers and cold coffee, dark epic digital painting, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated blue accent #3d8fd6, painterly brushstrokes, seinen atmosphere --ar 4:5 --no neon everywhere, rainbow colors, text, watermark</t>
+          <t>holographic briefing table projecting layered maps of seven different historical eras, gloved hands of unseen officers pointing at a blank unmapped region, dark war-room of the RIKKEN facility, papers and cold coffee, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated blue accent #3d8fd6, seinen atmosphere --no neon everywhere, rainbow colors, text, watermark</t>
         </is>
       </c>
     </row>
@@ -1361,7 +1361,7 @@
       </c>
       <c r="S10" s="5" t="inlineStr">
         <is>
-          <t>young franco-senegalese woman medic in a sleek black biotech suit, thin cyan nano-fluid conduits glowing along her forearms, open palm with fine diffuser pores emitting soft cyan light, clinical calm expression, dark field-hospital corner of a mission camp, subject centered upper half, dark epic digital painting, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated cyan accent, painterly, seinen atmosphere --ar 4:5 --no neon everywhere, rainbow colors, iron man style, text, watermark</t>
+          <t>young franco-senegalese woman medic in a sleek black biotech suit, thin cyan nano-fluid conduits glowing along her forearms, open palm with fine diffuser pores emitting soft cyan light, clinical calm expression, dark field-hospital corner of a mission camp, subject centered upper half, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated cyan accent, seinen atmosphere --no neon everywhere, rainbow colors, iron man style, text, watermark</t>
         </is>
       </c>
     </row>
@@ -1446,7 +1446,7 @@
       </c>
       <c r="S11" s="5" t="inlineStr">
         <is>
-          <t>young japanese woman in a sleek dark biotech suit, fine fractal sensor lines glowing deep blue across her forearms, extended HUD visor over her eyes reflecting cascading probability data, hyper-focused expression, dark analysis chamber, subject centered upper half, dark epic digital painting, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated deep blue accent, painterly brushstrokes, seinen atmosphere --ar 4:5 --no neon everywhere, rainbow colors, cyberpunk pink purple, text, watermark</t>
+          <t>young japanese woman in a sleek dark biotech suit, fine fractal sensor lines glowing deep blue across her forearms, extended HUD visor over her eyes reflecting cascading probability data, hyper-focused expression, dark analysis chamber, subject centered upper half, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated deep blue accent, seinen atmosphere --no neon everywhere, rainbow colors, cyberpunk pink purple, text, watermark</t>
         </is>
       </c>
     </row>
@@ -1513,7 +1513,7 @@
       </c>
       <c r="S12" s="5" t="inlineStr">
         <is>
-          <t>male traveler in a sleek dark biotech suit with contained ember-like combustion channels along arms and shoulders, heat shimmer rising from his gauntlets, embers drifting in a dark testing chamber, controlled and calm, no flames raging, subject centered upper half, dark epic digital painting, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated ember orange-red accent, painterly, seinen atmosphere --ar 4:5 --no neon everywhere, rainbow colors, fire everywhere, iron man style, text, watermark</t>
+          <t>male traveler in a sleek dark biotech suit with contained ember-like combustion channels along arms and shoulders, heat shimmer rising from his gauntlets, embers drifting in a dark testing chamber, controlled and calm, no flames raging, subject centered upper half, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated ember orange-red accent, seinen atmosphere --no neon everywhere, rainbow colors, fire everywhere, iron man style, text, watermark</t>
         </is>
       </c>
     </row>
@@ -1596,7 +1596,7 @@
       </c>
       <c r="S13" s="5" t="inlineStr">
         <is>
-          <t>veteran escort traveler in a heavy dark biotech suit with thick worn plates and old mission scars on the armor, standing protectively in a doorway of black metal, grey temples, tired unshakable eyes, faint blue light lines, subject centered upper half, dark epic digital painting, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated blue accent #3d8fd6, painterly brushstrokes, seinen atmosphere --ar 4:5 --no neon everywhere, rainbow colors, iron man style, text, watermark</t>
+          <t>veteran escort traveler in a heavy dark biotech suit with thick worn plates and old mission scars on the armor, standing protectively in a doorway of black metal, grey temples, tired unshakable eyes, faint blue light lines, subject centered upper half, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated blue accent #3d8fd6, seinen atmosphere --no neon everywhere, rainbow colors, iron man style, text, watermark</t>
         </is>
       </c>
     </row>
@@ -1671,7 +1671,7 @@
       </c>
       <c r="S14" s="5" t="inlineStr">
         <is>
-          <t>traveler mid-dematerialization into blue-white light lines while reaching desperately toward the viewer, dark collapsed historical ruin around, dust and debris frozen mid-air, urgency and rescue, dark epic digital painting, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated blue accent #3d8fd6, painterly, seinen atmosphere --ar 4:5 --no neon everywhere, rainbow colors, text, watermark</t>
+          <t>traveler mid-dematerialization into blue-white light lines while reaching desperately toward the viewer, dark collapsed historical ruin around, dust and debris frozen mid-air, urgency and rescue, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated blue accent #3d8fd6, seinen atmosphere --no neon everywhere, rainbow colors, text, watermark</t>
         </is>
       </c>
     </row>
@@ -1746,7 +1746,7 @@
       </c>
       <c r="S15" s="5" t="inlineStr">
         <is>
-          <t>translucent geometric energy dome protecting a squad of dark-suited travelers kneeling on a transfer platform, impacts flaring softly on the dome surface, dark hall beyond, the dome light is faint blue and contained, dark epic digital painting, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated blue accent #3d8fd6, painterly brushstrokes, seinen atmosphere --ar 4:5 --no neon everywhere, rainbow colors, text, watermark</t>
+          <t>translucent geometric energy dome protecting a squad of dark-suited travelers kneeling on a transfer platform, impacts flaring softly on the dome surface, dark hall beyond, the dome light is faint blue and contained, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated blue accent #3d8fd6, seinen atmosphere --no neon everywhere, rainbow colors, text, watermark</t>
         </is>
       </c>
     </row>
@@ -1813,7 +1813,7 @@
       </c>
       <c r="S16" s="5" t="inlineStr">
         <is>
-          <t>female squad coordinator in dark RIKKEN officer uniform standing before a wall of mission screens showing three teams in different eras, headset on, one hand raised mid-order, dark control room lit by pale blue monitors, subject centered upper half, dark epic digital painting, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated blue accent #3d8fd6, painterly, seinen atmosphere --ar 4:5 --no neon everywhere, rainbow colors, text, watermark</t>
+          <t>female squad coordinator in dark RIKKEN officer uniform standing before a wall of mission screens showing three teams in different eras, headset on, one hand raised mid-order, dark control room lit by pale blue monitors, subject centered upper half, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated blue accent #3d8fd6, seinen atmosphere --no neon everywhere, rainbow colors, text, watermark</t>
         </is>
       </c>
     </row>
@@ -1902,7 +1902,7 @@
       </c>
       <c r="S17" s="5" t="inlineStr">
         <is>
-          <t>young russian man with insolent grin mid-parkour leap across dark rooftops, sleek black biotech suit with visible nitro thrusters on calves and back glowing warm orange, aerodynamic panels retracting, motion energy, subject centered upper half, dark epic digital painting, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated warm orange accent, contained light lines, painterly, seinen atmosphere --ar 4:5 --no neon everywhere, rainbow colors, iron man style, text, watermark</t>
+          <t>young russian man with insolent grin mid-parkour leap across dark rooftops, sleek black biotech suit with visible nitro thrusters on calves and back glowing warm orange, aerodynamic panels retracting, motion energy, subject centered upper half, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated warm orange accent, contained light lines, seinen atmosphere --no neon everywhere, rainbow colors, iron man style, text, watermark</t>
         </is>
       </c>
     </row>
@@ -1987,7 +1987,7 @@
       </c>
       <c r="S18" s="5" t="inlineStr">
         <is>
-          <t>traveler in a sleek dark biotech suit standing in a foggy historical battlefield, rusted iron debris and broken blades levitating in a slow orbit around him, faint magnetic field distortion, contained pale blue light lines on his suit, subject centered upper half, dark epic digital painting, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated blue accent #3d8fd6, painterly brushstrokes, seinen atmosphere --ar 4:5 --no neon everywhere, rainbow colors, iron man style, text, watermark</t>
+          <t>traveler in a sleek dark biotech suit standing in a foggy historical battlefield, rusted iron debris and broken blades levitating in a slow orbit around him, faint magnetic field distortion, contained pale blue light lines on his suit, subject centered upper half, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated blue accent #3d8fd6, seinen atmosphere --no neon everywhere, rainbow colors, iron man style, text, watermark</t>
         </is>
       </c>
     </row>
@@ -2062,7 +2062,7 @@
       </c>
       <c r="S19" s="5" t="inlineStr">
         <is>
-          <t>the massive spherical energy core of the RIKKEN central deep under Odaiba surging with blue-white power, catwalks and tiny engineer silhouettes dwarfed by the machine, conduits blazing with contained light, industrial cathedral scale, dark epic digital painting, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated blue accent #3d8fd6, painterly, seinen atmosphere --ar 4:5 --no neon everywhere, rainbow colors, explosion, text, watermark</t>
+          <t>the massive spherical energy core of the RIKKEN central deep under Odaiba surging with blue-white power, catwalks and tiny engineer silhouettes dwarfed by the machine, conduits blazing with contained light, industrial cathedral scale, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated blue accent #3d8fd6, seinen atmosphere --no neon everywhere, rainbow colors, explosion, text, watermark</t>
         </is>
       </c>
     </row>
@@ -2129,7 +2129,7 @@
       </c>
       <c r="S20" s="5" t="inlineStr">
         <is>
-          <t>stern japanese woman in her fifties in an impeccable dark RIKKEN uniform, seated alone at an elevated jury desk in the white immaculate test center, arms crossed, evaluating gaze cutting downward at the viewer, clinical white light, one blue insignia, subject centered upper half, dark epic digital painting, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated blue accent #3d8fd6, painterly, seinen atmosphere --ar 4:5 --no neon everywhere, rainbow colors, text, watermark</t>
+          <t>stern japanese woman in her fifties in an impeccable dark RIKKEN uniform, seated alone at an elevated jury desk in the white immaculate test center, arms crossed, evaluating gaze cutting downward at the viewer, clinical white light, one blue insignia, subject centered upper half, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated blue accent #3d8fd6, seinen atmosphere --no neon everywhere, rainbow colors, text, watermark</t>
         </is>
       </c>
     </row>
@@ -2218,7 +2218,7 @@
       </c>
       <c r="S21" s="5" t="inlineStr">
         <is>
-          <t>imposing japanese man in his sixties, granite face and grey brush cut, wearing a first-generation biotech suit with visible patinated copper and brass conductors, thick old-school plates, mechanical piston joints, standing like a rock in a dark hangar, quiet overwhelming aura, subject centered upper half, dark epic digital painting, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated warm brass accent, painterly, seinen atmosphere --ar 4:5 --no neon everywhere, rainbow colors, iron man style, text, watermark</t>
+          <t>imposing japanese man in his sixties, granite face and grey brush cut, wearing a first-generation biotech suit with visible patinated copper and brass conductors, thick old-school plates, mechanical piston joints, standing like a rock in a dark hangar, quiet overwhelming aura, subject centered upper half, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated warm brass accent, seinen atmosphere --no neon everywhere, rainbow colors, iron man style, text, watermark</t>
         </is>
       </c>
     </row>
@@ -2285,7 +2285,7 @@
       </c>
       <c r="S22" s="5" t="inlineStr">
         <is>
-          <t>broad-shouldered chinese man in a heavy dark biotech suit, forearm and chest plates condensing into matte-black liquid-stone density, one massive fist wrapped in a compressive distortion aura, cracked concrete under his feet, dark testing arena, subject centered upper half, dark epic digital painting, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated blue accent #3d8fd6, painterly brushstrokes, seinen atmosphere --ar 4:5 --no neon everywhere, rainbow colors, hulk, giant mecha, text, watermark</t>
+          <t>broad-shouldered chinese man in a heavy dark biotech suit, forearm and chest plates condensing into matte-black liquid-stone density, one massive fist wrapped in a compressive distortion aura, cracked concrete under his feet, dark testing arena, subject centered upper half, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated blue accent #3d8fd6, seinen atmosphere --no neon everywhere, rainbow colors, hulk, giant mecha, text, watermark</t>
         </is>
       </c>
     </row>
@@ -2374,7 +2374,7 @@
       </c>
       <c r="S23" s="5" t="inlineStr">
         <is>
-          <t>19 year old slim french-japanese young man, light beige tousled hair with dark strands and one single vivid red strand over his right brow, thin scar on right cheekbone, grey almond eyes, wearing a sleek black prototype biotech suit with modular reconfiguring panels, a small engraved golden circle glowing softly on his chest, faint multi-hued light lines syncing along his arms, dark platform hall, subject centered upper half, dark epic digital painting, dramatic chiaroscuro lighting, muted monochrome palette with red strand and golden circle as only accents, painterly, seinen atmosphere --ar 4:5 --no neon everywhere, rainbow colors, iron man style, text, watermark</t>
+          <t>19 year old slim french-japanese young man, light beige tousled hair with dark strands and one single vivid red strand over his right brow, thin scar on right cheekbone, grey almond eyes, wearing a sleek black prototype biotech suit with modular reconfiguring panels, a small engraved golden circle glowing softly on his chest, faint multi-hued light lines syncing along his arms, dark platform hall, subject centered upper half, dramatic chiaroscuro lighting, muted monochrome palette with red strand and golden circle as only accents, seinen atmosphere --no neon everywhere, rainbow colors, iron man style, text, watermark</t>
         </is>
       </c>
     </row>
@@ -2457,7 +2457,7 @@
       </c>
       <c r="S24" s="5" t="inlineStr">
         <is>
-          <t>unremarkable middle-aged agent in a dark RIKKEN staff uniform standing in a facility corridor at 3am, authentic institute badge on his chest, half of his face swallowed by shadow, the other half perfectly ordinary, one tiny red LED reflected in his eye, subject centered upper half, dark epic digital painting, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated red accent #c23b4e, painterly, seinen atmosphere --ar 4:5 --no neon everywhere, rainbow colors, text, watermark</t>
+          <t>unremarkable middle-aged agent in a dark RIKKEN staff uniform standing in a facility corridor at 3am, authentic institute badge on his chest, half of his face swallowed by shadow, the other half perfectly ordinary, one tiny red LED reflected in his eye, subject centered upper half, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated red accent #c23b4e, seinen atmosphere --no neon everywhere, rainbow colors, text, watermark</t>
         </is>
       </c>
     </row>
@@ -2524,7 +2524,7 @@
       </c>
       <c r="S25" s="5" t="inlineStr">
         <is>
-          <t>young candidate in recruit fatigues standing in line at the white RIKKEN test center, posture identical to the others but eyes measuring the room like a professional, faint red thread bracelet under his sleeve, clinical white light, half his face in shadow, subject centered upper half, dark epic digital painting, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated red accent #c23b4e, painterly, seinen atmosphere --ar 4:5 --no neon everywhere, rainbow colors, text, watermark</t>
+          <t>young candidate in recruit fatigues standing in line at the white RIKKEN test center, posture identical to the others but eyes measuring the room like a professional, faint red thread bracelet under his sleeve, clinical white light, half his face in shadow, subject centered upper half, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated red accent #c23b4e, seinen atmosphere --no neon everywhere, rainbow colors, text, watermark</t>
         </is>
       </c>
     </row>
@@ -2591,7 +2591,7 @@
       </c>
       <c r="S26" s="5" t="inlineStr">
         <is>
-          <t>operative in a stolen dark biotech suit moving silently through an empty facility corridor at night, suit light lines flickering red and miscalibrated, one hand trailing along the wall, security camera dead behind him, subject centered upper half, dark epic digital painting, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated red accent #c23b4e, contained light lines, painterly, seinen atmosphere --ar 4:5 --no neon everywhere, rainbow colors, iron man style, text, watermark</t>
+          <t>operative in a stolen dark biotech suit moving silently through an empty facility corridor at night, suit light lines flickering red and miscalibrated, one hand trailing along the wall, security camera dead behind him, subject centered upper half, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated red accent #c23b4e, contained light lines, seinen atmosphere --no neon everywhere, rainbow colors, iron man style, text, watermark</t>
         </is>
       </c>
     </row>
@@ -2658,7 +2658,7 @@
       </c>
       <c r="S27" s="5" t="inlineStr">
         <is>
-          <t>watcher in dark civilian clothes standing on a rooftop overlooking Tokyo bay at night, binoculars lowered, patient posture, the city lights muted and grey except one distant red aircraft beacon, wind in his coat, subject centered upper half, dark epic digital painting, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated red accent #c23b4e, painterly brushstrokes, seinen atmosphere --ar 4:5 --no neon everywhere, rainbow colors, cyberpunk, text, watermark</t>
+          <t>watcher in dark civilian clothes standing on a rooftop overlooking Tokyo bay at night, binoculars lowered, patient posture, the city lights muted and grey except one distant red aircraft beacon, wind in his coat, subject centered upper half, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated red accent #c23b4e, seinen atmosphere --no neon everywhere, rainbow colors, cyberpunk, text, watermark</t>
         </is>
       </c>
     </row>
@@ -2741,7 +2741,7 @@
       </c>
       <c r="S28" s="5" t="inlineStr">
         <is>
-          <t>kairos fighter in a mismatched stolen biotech suit, panels from different CELL generations bolted together, red light lines sputtering and glitching at the seams, aggressive hunched stance in a dark parking structure, subject centered upper half, dark epic digital painting, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated red accent #c23b4e, painterly, seinen atmosphere --ar 4:5 --no neon everywhere, rainbow colors, iron man style, text, watermark</t>
+          <t>kairos fighter in a mismatched stolen biotech suit, panels from different CELL generations bolted together, red light lines sputtering and glitching at the seams, aggressive hunched stance in a dark parking structure, subject centered upper half, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated red accent #c23b4e, seinen atmosphere --no neon everywhere, rainbow colors, iron man style, text, watermark</t>
         </is>
       </c>
     </row>
@@ -2808,7 +2808,7 @@
       </c>
       <c r="S29" s="5" t="inlineStr">
         <is>
-          <t>cold professional woman in a tailored dark coat standing over an open briefcase of precise tech instruments, surgical calm, dark hotel room with Tokyo night skyline muted behind glass, one red instrument light, subject centered upper half, dark epic digital painting, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated red accent #c23b4e, painterly brushstrokes, seinen atmosphere --ar 4:5 --no neon everywhere, rainbow colors, blood, text, watermark</t>
+          <t>cold professional woman in a tailored dark coat standing over an open briefcase of precise tech instruments, surgical calm, dark hotel room with Tokyo night skyline muted behind glass, one red instrument light, subject centered upper half, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated red accent #c23b4e, seinen atmosphere --no neon everywhere, rainbow colors, blood, text, watermark</t>
         </is>
       </c>
     </row>
@@ -2875,7 +2875,7 @@
       </c>
       <c r="S30" s="5" t="inlineStr">
         <is>
-          <t>executive in an impeccable suit standing in a glass corner office above Tokyo at night, back to the viewer, reflection in the window showing a face we cannot quite read, red seal stamp resting on signed documents, subject centered upper half, dark epic digital painting, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated red accent #c23b4e, painterly, seinen atmosphere --ar 4:5 --no neon everywhere, rainbow colors, text, watermark</t>
+          <t>executive in an impeccable suit standing in a glass corner office above Tokyo at night, back to the viewer, reflection in the window showing a face we cannot quite read, red seal stamp resting on signed documents, subject centered upper half, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated red accent #c23b4e, seinen atmosphere --no neon everywhere, rainbow colors, text, watermark</t>
         </is>
       </c>
     </row>
@@ -2942,7 +2942,7 @@
       </c>
       <c r="S31" s="5" t="inlineStr">
         <is>
-          <t>close-up of a gloved hand sliding a thin red-sealed dossier across a polished dark table toward a trembling bare hand, tea untouched, faces out of frame, dark meeting room, the seal is the only color, dark epic digital painting, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated red accent #c23b4e, painterly brushstrokes, seinen atmosphere --ar 4:5 --no neon everywhere, rainbow colors, text, watermark</t>
+          <t>close-up of a gloved hand sliding a thin red-sealed dossier across a polished dark table toward a trembling bare hand, tea untouched, faces out of frame, dark meeting room, the seal is the only color, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated red accent #c23b4e, seinen atmosphere --no neon everywhere, rainbow colors, text, watermark</t>
         </is>
       </c>
     </row>
@@ -3009,7 +3009,7 @@
       </c>
       <c r="S32" s="5" t="inlineStr">
         <is>
-          <t>circular time-transfer platform short-circuiting in a dark hall, its blue ring guttering out while thin red warning strobes sweep the walls, sparks raining, a small sabotage device blinking red at the platform base, no people, dark epic digital painting, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated red accent #c23b4e, painterly, seinen atmosphere --ar 4:5 --no neon everywhere, rainbow colors, explosion, text, watermark</t>
+          <t>circular time-transfer platform short-circuiting in a dark hall, its blue ring guttering out while thin red warning strobes sweep the walls, sparks raining, a small sabotage device blinking red at the platform base, no people, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated red accent #c23b4e, seinen atmosphere --no neon everywhere, rainbow colors, explosion, text, watermark</t>
         </is>
       </c>
     </row>
@@ -3076,7 +3076,7 @@
       </c>
       <c r="S33" s="5" t="inlineStr">
         <is>
-          <t>female kairos operative in a dark tech coat raising a small parasite emitter, translucent red interference waves rippling from it, a distant traveler's suit light lines visibly stuttering and dying, dark facility hall, subject centered upper half, dark epic digital painting, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated red accent #c23b4e, painterly, seinen atmosphere --ar 4:5 --no neon everywhere, rainbow colors, text, watermark</t>
+          <t>female kairos operative in a dark tech coat raising a small parasite emitter, translucent red interference waves rippling from it, a distant traveler's suit light lines visibly stuttering and dying, dark facility hall, subject centered upper half, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated red accent #c23b4e, seinen atmosphere --no neon everywhere, rainbow colors, text, watermark</t>
         </is>
       </c>
     </row>
@@ -3143,7 +3143,7 @@
       </c>
       <c r="S34" s="5" t="inlineStr">
         <is>
-          <t>lean duelist in a stolen sleek biotech suit, contained electric arcs crawling between his gauntlets, red-tinged capacitor lines pulsing unstably along his spine, combat stance in a rain-slick dark alley, subject centered upper half, dark epic digital painting, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated red accent #c23b4e, painterly brushstrokes, seinen atmosphere --ar 4:5 --no neon everywhere, rainbow colors, lightning storm, iron man style, text, watermark</t>
+          <t>lean duelist in a stolen sleek biotech suit, contained electric arcs crawling between his gauntlets, red-tinged capacitor lines pulsing unstably along his spine, combat stance in a rain-slick dark alley, subject centered upper half, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated red accent #c23b4e, seinen atmosphere --no neon everywhere, rainbow colors, lightning storm, iron man style, text, watermark</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3210,7 @@
       </c>
       <c r="S35" s="5" t="inlineStr">
         <is>
-          <t>charming recruiter in RIKKEN colors leaning across an interview table toward an unseen candidate, warm practiced smile that stops below the eyes, red pen turning slowly between his fingers, dark interview room, subject centered upper half, dark epic digital painting, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated red accent #c23b4e, painterly, seinen atmosphere --ar 4:5 --no neon everywhere, rainbow colors, text, watermark</t>
+          <t>charming recruiter in RIKKEN colors leaning across an interview table toward an unseen candidate, warm practiced smile that stops below the eyes, red pen turning slowly between his fingers, dark interview room, subject centered upper half, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated red accent #c23b4e, seinen atmosphere --no neon everywhere, rainbow colors, text, watermark</t>
         </is>
       </c>
     </row>
@@ -3277,7 +3277,7 @@
       </c>
       <c r="S36" s="5" t="inlineStr">
         <is>
-          <t>huge enforcer in a reinforced dark suit filling a narrow basement corridor of the facility, head bowed under the ceiling, knuckles wrapped in red-lit compression bands, pipes and steam around him, subject centered upper half, dark epic digital painting, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated red accent #c23b4e, painterly brushstrokes, seinen atmosphere --ar 4:5 --no neon everywhere, rainbow colors, hulk, giant mecha, text, watermark</t>
+          <t>huge enforcer in a reinforced dark suit filling a narrow basement corridor of the facility, head bowed under the ceiling, knuckles wrapped in red-lit compression bands, pipes and steam around him, subject centered upper half, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated red accent #c23b4e, seinen atmosphere --no neon everywhere, rainbow colors, hulk, giant mecha, text, watermark</t>
         </is>
       </c>
     </row>
@@ -3344,7 +3344,7 @@
       </c>
       <c r="S37" s="5" t="inlineStr">
         <is>
-          <t>a traveler's biotech suit mid-activation abruptly failing, its blue light lines shattering into static as a translucent red interference wave passes through the frame, the traveler's silhouette frozen mid-gesture in a dark hall, dark epic digital painting, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated red accent #c23b4e, painterly, seinen atmosphere --ar 4:5 --no neon everywhere, rainbow colors, text, watermark</t>
+          <t>a traveler's biotech suit mid-activation abruptly failing, its blue light lines shattering into static as a translucent red interference wave passes through the frame, the traveler's silhouette frozen mid-gesture in a dark hall, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated red accent #c23b4e, seinen atmosphere --no neon everywhere, rainbow colors, text, watermark</t>
         </is>
       </c>
     </row>
@@ -3411,7 +3411,7 @@
       </c>
       <c r="S38" s="5" t="inlineStr">
         <is>
-          <t>human figure being torn backward out of a historical scene into red-black static, the scene itself continuing undisturbed around the void he leaves, fingers clawing at air, sense of violent temporal removal, dark epic digital painting, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated red accent #c23b4e, painterly brushstrokes, seinen atmosphere --ar 4:5 --no neon everywhere, rainbow colors, gore, text, watermark</t>
+          <t>human figure being torn backward out of a historical scene into red-black static, the scene itself continuing undisturbed around the void he leaves, fingers clawing at air, sense of violent temporal removal, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated red accent #c23b4e, seinen atmosphere --no neon everywhere, rainbow colors, gore, text, watermark</t>
         </is>
       </c>
     </row>
@@ -3478,7 +3478,7 @@
       </c>
       <c r="S39" s="5" t="inlineStr">
         <is>
-          <t>female kairos agent in a stolen suit kneeling in a foggy blind-zone battlefield, prying a relic from the mud into a red-lit containment case, disturbed historical dead around her under the mist, disrespectful haste, subject centered upper half, dark epic digital painting, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated red accent #c23b4e, painterly, seinen atmosphere --ar 4:5 --no neon everywhere, rainbow colors, gore, text, watermark</t>
+          <t>female kairos agent in a stolen suit kneeling in a foggy blind-zone battlefield, prying a relic from the mud into a red-lit containment case, disturbed historical dead around her under the mist, disrespectful haste, subject centered upper half, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated red accent #c23b4e, seinen atmosphere --no neon everywhere, rainbow colors, gore, text, watermark</t>
         </is>
       </c>
     </row>
@@ -3545,7 +3545,7 @@
       </c>
       <c r="S40" s="5" t="inlineStr">
         <is>
-          <t>interrogator in an immaculate dark uniform standing beside an empty steel chair in a blinding white interrogation room, one red recording light on the wall, his shadow falling across the chair, quiet menace, subject centered upper half, dark epic digital painting, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated red accent #c23b4e, painterly brushstrokes, seinen atmosphere --ar 4:5 --no neon everywhere, rainbow colors, text, watermark</t>
+          <t>interrogator in an immaculate dark uniform standing beside an empty steel chair in a blinding white interrogation room, one red recording light on the wall, his shadow falling across the chair, quiet menace, subject centered upper half, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated red accent #c23b4e, seinen atmosphere --no neon everywhere, rainbow colors, text, watermark</t>
         </is>
       </c>
     </row>
@@ -3612,7 +3612,7 @@
       </c>
       <c r="S41" s="5" t="inlineStr">
         <is>
-          <t>kairos operative in a sleek stolen biotech suit standing calmly while a swarm of palm-sized drones orbits him in a slow red-lit constellation, each drone eye a tiny red point, dark server hall, subject centered upper half, dark epic digital painting, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated red accent #c23b4e, contained light lines, painterly, seinen atmosphere --ar 4:5 --no neon everywhere, rainbow colors, iron man style, text, watermark</t>
+          <t>kairos operative in a sleek stolen biotech suit standing calmly while a swarm of palm-sized drones orbits him in a slow red-lit constellation, each drone eye a tiny red point, dark server hall, subject centered upper half, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated red accent #c23b4e, contained light lines, seinen atmosphere --no neon everywhere, rainbow colors, iron man style, text, watermark</t>
         </is>
       </c>
     </row>
@@ -3679,7 +3679,7 @@
       </c>
       <c r="S42" s="5" t="inlineStr">
         <is>
-          <t>monumental cracked clock face suspended in darkness, thin red light bleeding through the fracture lines, a single silhouette stepping through the largest crack as through a door, shards of time frozen around, dark epic digital painting, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated red accent #c23b4e, painterly brushstrokes, seinen atmosphere --ar 4:5 --no neon everywhere, rainbow colors, text, watermark</t>
+          <t>monumental cracked clock face suspended in darkness, thin red light bleeding through the fracture lines, a single silhouette stepping through the largest crack as through a door, shards of time frozen around, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated red accent #c23b4e, seinen atmosphere --no neon everywhere, rainbow colors, text, watermark</t>
         </is>
       </c>
     </row>
@@ -3762,7 +3762,7 @@
       </c>
       <c r="S43" s="5" t="inlineStr">
         <is>
-          <t>distinguished japanese director in his fifties in a flawless dark suit, seated at a directorial desk high above Tokyo night, hands calmly folded, wearing a warm gentle smile that is slightly too perfect to be true, red seal ring on his finger, soft office light, subject centered upper half, dark epic digital painting, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated red accent #c23b4e, painterly, seinen atmosphere --ar 4:5 --no neon everywhere, rainbow colors, villain sneer, text, watermark</t>
+          <t>distinguished japanese director in his fifties in a flawless dark suit, seated at a directorial desk high above Tokyo night, hands calmly folded, wearing a warm gentle smile that is slightly too perfect to be true, red seal ring on his finger, soft office light, subject centered upper half, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated red accent #c23b4e, seinen atmosphere --no neon everywhere, rainbow colors, villain sneer, text, watermark</t>
         </is>
       </c>
     </row>
@@ -3829,7 +3829,7 @@
       </c>
       <c r="S44" s="5" t="inlineStr">
         <is>
-          <t>austere woman in a dark tailored suit standing in a shadowed archive of ledgers and red-stamped files, holding a single page up to a thin blade of light, faces of debtors pinned on threads behind her like a silent web, subject centered upper half, dark epic digital painting, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated red accent #c23b4e, painterly brushstrokes, seinen atmosphere --ar 4:5 --no neon everywhere, rainbow colors, text, watermark</t>
+          <t>austere woman in a dark tailored suit standing in a shadowed archive of ledgers and red-stamped files, holding a single page up to a thin blade of light, faces of debtors pinned on threads behind her like a silent web, subject centered upper half, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated red accent #c23b4e, seinen atmosphere --no neon everywhere, rainbow colors, text, watermark</t>
         </is>
       </c>
     </row>
@@ -3918,7 +3918,7 @@
       </c>
       <c r="S45" s="5" t="inlineStr">
         <is>
-          <t>gaunt japanese man with hollow calm eyes in a matte black biotech suit, thin prismatic conductor panels shimmering faintly across shoulders and forearms, twin adaptive blades half-extended from his forearms catching a red emergency light, empty facility hall at night, subject centered upper half, dark epic digital painting, dramatic chiaroscuro lighting, muted monochrome palette with prismatic shimmer and single red accent #c23b4e, painterly, seinen atmosphere --ar 4:5 --no neon everywhere, rainbow colors everywhere, iron man style, text, watermark</t>
+          <t>gaunt japanese man with hollow calm eyes in a matte black biotech suit, thin prismatic conductor panels shimmering faintly across shoulders and forearms, twin adaptive blades half-extended from his forearms catching a red emergency light, empty facility hall at night, subject centered upper half, dramatic chiaroscuro lighting, muted monochrome palette with prismatic shimmer and single red accent #c23b4e, seinen atmosphere --no neon everywhere, rainbow colors everywhere, iron man style, text, watermark</t>
         </is>
       </c>
     </row>
@@ -3985,7 +3985,7 @@
       </c>
       <c r="S46" s="5" t="inlineStr">
         <is>
-          <t>street kid in patched wool clothes and oversized cap standing in a fog-drowned parisian alley in 1888, iron scaffolding of a construction site looming as vague shapes in the mist behind, sharp knowing eyes, bronze sepia tones, the fog erasing every landmark, subject centered upper half, dark epic digital painting, dramatic chiaroscuro lighting, muted monochrome palette with a single warm bronze accent #b08d57, painterly brushstrokes, seinen atmosphere --ar 4:5 --no eiffel tower recognizable, rainbow colors, text, watermark</t>
+          <t>street kid in patched wool clothes and oversized cap standing in a fog-drowned parisian alley in 1888, iron scaffolding of a construction site looming as vague shapes in the mist behind, sharp knowing eyes, bronze sepia tones, the fog erasing every landmark, subject centered upper half, dramatic chiaroscuro lighting, muted monochrome palette with a single warm bronze accent #b08d57, seinen atmosphere --no eiffel tower recognizable, rainbow colors, text, watermark</t>
         </is>
       </c>
     </row>
@@ -4052,7 +4052,7 @@
       </c>
       <c r="S47" s="5" t="inlineStr">
         <is>
-          <t>laundress in rough 19th century workclothes wringing linen at a river bank at dawn, thick fog hiding the far shore and every monument, her breath visible, strong tired hands, warm bronze light through the mist, subject centered upper half, dark epic digital painting, dramatic chiaroscuro lighting, muted monochrome palette with a single warm bronze accent #b08d57, painterly brushstrokes, seinen atmosphere --ar 4:5 --no recognizable landmarks, rainbow colors, text, watermark</t>
+          <t>laundress in rough 19th century workclothes wringing linen at a river bank at dawn, thick fog hiding the far shore and every monument, her breath visible, strong tired hands, warm bronze light through the mist, subject centered upper half, dramatic chiaroscuro lighting, muted monochrome palette with a single warm bronze accent #b08d57, seinen atmosphere --no recognizable landmarks, rainbow colors, text, watermark</t>
         </is>
       </c>
     </row>
@@ -4127,7 +4127,7 @@
       </c>
       <c r="S48" s="5" t="inlineStr">
         <is>
-          <t>masterless samurai in worn dark travel clothes standing at the foot of a wooden bridge swallowed by river mist, hand resting on a chipped saya, the far end of the bridge invisible, no banners no crest, flood-heavy river below, subject centered upper half, dark epic digital painting, dramatic chiaroscuro lighting, muted monochrome palette with a single warm bronze accent #b08d57, painterly brushstrokes, seinen atmosphere --ar 4:5 --no famous castle, rainbow colors, text, watermark</t>
+          <t>masterless samurai in worn dark travel clothes standing at the foot of a wooden bridge swallowed by river mist, hand resting on a chipped saya, the far end of the bridge invisible, no banners no crest, flood-heavy river below, subject centered upper half, dramatic chiaroscuro lighting, muted monochrome palette with a single warm bronze accent #b08d57, seinen atmosphere --no famous castle, rainbow colors, text, watermark</t>
         </is>
       </c>
     </row>
@@ -4194,7 +4194,7 @@
       </c>
       <c r="S49" s="5" t="inlineStr">
         <is>
-          <t>weathered stonemason in medieval work clothes laying stones of a small unfinished mountain chapel as snow begins to bury the pass, wooden scaffold creaking in the wind, mallet in cracked hands, whiteout erasing the valley below, subject centered upper half, dark epic digital painting, dramatic chiaroscuro lighting, muted monochrome palette with a single warm bronze accent #b08d57, painterly, seinen atmosphere --ar 4:5 --no recognizable cathedral, rainbow colors, text, watermark</t>
+          <t>weathered stonemason in medieval work clothes laying stones of a small unfinished mountain chapel as snow begins to bury the pass, wooden scaffold creaking in the wind, mallet in cracked hands, whiteout erasing the valley below, subject centered upper half, dramatic chiaroscuro lighting, muted monochrome palette with a single warm bronze accent #b08d57, seinen atmosphere --no recognizable cathedral, rainbow colors, text, watermark</t>
         </is>
       </c>
     </row>
@@ -4261,7 +4261,7 @@
       </c>
       <c r="S50" s="5" t="inlineStr">
         <is>
-          <t>lone roman legionary in mud-caked worn armor standing in a dark primeval forest, shield split, fog between colossal trees swallowing the rest of his column, no standard visible, exhausted defiance, moss and rain, subject centered upper half, dark epic digital painting, dramatic chiaroscuro lighting, muted monochrome palette with a single warm bronze accent #b08d57, painterly brushstrokes, seinen atmosphere --ar 4:5 --no roman monument, rainbow colors, text, watermark</t>
+          <t>lone roman legionary in mud-caked worn armor standing in a dark primeval forest, shield split, fog between colossal trees swallowing the rest of his column, no standard visible, exhausted defiance, moss and rain, subject centered upper half, dramatic chiaroscuro lighting, muted monochrome palette with a single warm bronze accent #b08d57, seinen atmosphere --no roman monument, rainbow colors, text, watermark</t>
         </is>
       </c>
     </row>
@@ -4328,7 +4328,7 @@
       </c>
       <c r="S51" s="5" t="inlineStr">
         <is>
-          <t>harpooner in heavy oilskins standing at the icy bow of a whaling boat locked in pack ice, harpoon planted, breath steaming, the sea and sky fused into one grey fog wall, frost in his beard, subject centered upper half, dark epic digital painting, dramatic chiaroscuro lighting, muted monochrome palette with a single warm bronze accent #b08d57, painterly brushstrokes, seinen atmosphere --ar 4:5 --no rainbow colors, text, watermark</t>
+          <t>harpooner in heavy oilskins standing at the icy bow of a whaling boat locked in pack ice, harpoon planted, breath steaming, the sea and sky fused into one grey fog wall, frost in his beard, subject centered upper half, dramatic chiaroscuro lighting, muted monochrome palette with a single warm bronze accent #b08d57, seinen atmosphere --no rainbow colors, text, watermark</t>
         </is>
       </c>
     </row>
@@ -4395,7 +4395,7 @@
       </c>
       <c r="S52" s="5" t="inlineStr">
         <is>
-          <t>colossal prehistoric steppe bear rearing in a blizzard on an endless white plain, fur crusted with ice, breath like smoke, its shape half-dissolved by the snowstorm that erases the horizon, primal and indifferent, subject centered upper half, dark epic digital painting, dramatic chiaroscuro lighting, muted monochrome palette with a single warm bronze accent #b08d57, painterly brushstrokes, seinen atmosphere --ar 4:5 --no rainbow colors, text, watermark</t>
+          <t>colossal prehistoric steppe bear rearing in a blizzard on an endless white plain, fur crusted with ice, breath like smoke, its shape half-dissolved by the snowstorm that erases the horizon, primal and indifferent, subject centered upper half, dramatic chiaroscuro lighting, muted monochrome palette with a single warm bronze accent #b08d57, seinen atmosphere --no rainbow colors, text, watermark</t>
         </is>
       </c>
     </row>
@@ -4462,7 +4462,7 @@
       </c>
       <c r="S53" s="5" t="inlineStr">
         <is>
-          <t>a bare human hand dissolving into drifting golden dust motes inside a single blade of late afternoon light, dark empty barn interior, the dust rising and scattering like memory, quiet and sad, dark epic digital painting, dramatic chiaroscuro lighting, muted monochrome palette with a single warm bronze accent #b08d57, painterly brushstrokes, seinen atmosphere --ar 4:5 --no rainbow colors, skeleton, text, watermark</t>
+          <t>a bare human hand dissolving into drifting golden dust motes inside a single blade of late afternoon light, dark empty barn interior, the dust rising and scattering like memory, quiet and sad, dramatic chiaroscuro lighting, muted monochrome palette with a single warm bronze accent #b08d57, seinen atmosphere --no rainbow colors, skeleton, text, watermark</t>
         </is>
       </c>
     </row>
@@ -4529,7 +4529,7 @@
       </c>
       <c r="S54" s="5" t="inlineStr">
         <is>
-          <t>crowded blurry historical tavern scene painted in motion, every figure slightly smeared except one perfectly sharp empty chair at the center table with a still-steaming cup before it, the absence louder than the crowd, dark epic digital painting, dramatic chiaroscuro lighting, muted monochrome palette with a single warm bronze accent #b08d57, painterly brushstrokes, seinen atmosphere --ar 4:5 --no rainbow colors, text, watermark</t>
+          <t>crowded blurry historical tavern scene, every figure slightly smeared except one perfectly sharp empty chair at the center table with a still-steaming cup before it, the absence louder than the crowd, dramatic chiaroscuro lighting, muted monochrome palette with a single warm bronze accent #b08d57, seinen atmosphere --no rainbow colors, text, watermark</t>
         </is>
       </c>
     </row>
@@ -4596,7 +4596,7 @@
       </c>
       <c r="S55" s="5" t="inlineStr">
         <is>
-          <t>barefoot young messenger girl sprinting through a narrow ancient market street before dawn, sealed letter clutched to her chest, dust rising behind her bare heels, awnings and shadows blurring past, no era landmark visible, subject centered upper half, dark epic digital painting, dramatic chiaroscuro lighting, muted monochrome palette with a single warm bronze accent #b08d57, painterly brushstrokes, seinen atmosphere --ar 4:5 --no rainbow colors, text, watermark</t>
+          <t>barefoot young messenger girl sprinting through a narrow ancient market street before dawn, sealed letter clutched to her chest, dust rising behind her bare heels, awnings and shadows blurring past, no era landmark visible, subject centered upper half, dramatic chiaroscuro lighting, muted monochrome palette with a single warm bronze accent #b08d57, seinen atmosphere --no rainbow colors, text, watermark</t>
         </is>
       </c>
     </row>
@@ -4663,7 +4663,7 @@
       </c>
       <c r="S56" s="5" t="inlineStr">
         <is>
-          <t>old griot storyteller mid-tale at a night fire, hands spread wide casting long shadows, circle of captivated listeners leaning in from the darkness, sparks rising like his words, no monument no writing anywhere, subject centered upper half, dark epic digital painting, dramatic chiaroscuro lighting, muted monochrome palette with a single warm bronze accent #b08d57, painterly brushstrokes, seinen atmosphere --ar 4:5 --no rainbow colors, text, watermark</t>
+          <t>old griot storyteller mid-tale at a night fire, hands spread wide casting long shadows, circle of captivated listeners leaning in from the darkness, sparks rising like his words, no monument no writing anywhere, subject centered upper half, dramatic chiaroscuro lighting, muted monochrome palette with a single warm bronze accent #b08d57, seinen atmosphere --no rainbow colors, text, watermark</t>
         </is>
       </c>
     </row>
@@ -4730,7 +4730,7 @@
       </c>
       <c r="S57" s="5" t="inlineStr">
         <is>
-          <t>mountain woman warrior in furs and iron standing alone in a snowstorm at a narrow alpine pass, long spear planted, the path behind her vanishing into whiteout, ice in her braids, immovable calm, subject centered upper half, dark epic digital painting, dramatic chiaroscuro lighting, muted monochrome palette with a single warm bronze accent #b08d57, painterly brushstrokes, seinen atmosphere --ar 4:5 --no rainbow colors, fantasy armor, text, watermark</t>
+          <t>mountain woman warrior in furs and iron standing alone in a snowstorm at a narrow alpine pass, long spear planted, the path behind her vanishing into whiteout, ice in her braids, immovable calm, subject centered upper half, dramatic chiaroscuro lighting, muted monochrome palette with a single warm bronze accent #b08d57, seinen atmosphere --no rainbow colors, fantasy armor, text, watermark</t>
         </is>
       </c>
     </row>
@@ -4797,7 +4797,7 @@
       </c>
       <c r="S58" s="5" t="inlineStr">
         <is>
-          <t>wide historical landscape whose center is simply unwritten, a soft void of raw canvas texture swallowing the middle of the scene, painted world fraying into nothing at its edges, birds flying around the absence, eerie and calm, dark epic digital painting, dramatic chiaroscuro lighting, muted monochrome palette with a single warm bronze accent #b08d57, painterly brushstrokes, seinen atmosphere --ar 4:5 --no rainbow colors, portal, text, watermark</t>
+          <t>wide historical landscape whose center is simply unwritten, a soft blank void swallowing the middle of the scene, the world fraying into nothing at its edges, birds flying around the absence, eerie and calm, dramatic chiaroscuro lighting, muted monochrome palette with a single warm bronze accent #b08d57, seinen atmosphere --no rainbow colors, portal, text, watermark</t>
         </is>
       </c>
     </row>
@@ -4864,7 +4864,7 @@
       </c>
       <c r="S59" s="5" t="inlineStr">
         <is>
-          <t>lean swordsman in dark simple garb waiting at the far end of a mist-drowned wooden bridge, blade still sheathed, one hand raised in silent invitation, river fog erasing everything beyond ten paces, coiled stillness, subject centered upper half, dark epic digital painting, dramatic chiaroscuro lighting, muted monochrome palette with a single warm bronze accent #b08d57, painterly brushstrokes, seinen atmosphere --ar 4:5 --no famous landmark, rainbow colors, text, watermark</t>
+          <t>lean swordsman in dark simple garb waiting at the far end of a mist-drowned wooden bridge, blade still sheathed, one hand raised in silent invitation, river fog erasing everything beyond ten paces, coiled stillness, subject centered upper half, dramatic chiaroscuro lighting, muted monochrome palette with a single warm bronze accent #b08d57, seinen atmosphere --no famous landmark, rainbow colors, text, watermark</t>
         </is>
       </c>
     </row>
@@ -4931,7 +4931,7 @@
       </c>
       <c r="S60" s="5" t="inlineStr">
         <is>
-          <t>early 1900s battleship emerging half-real from a wall of sea fog, hull streaked with rust, gun turrets silent, no flag identifiable, the fog actively swallowing its stern as if unwriting it, cold heavy sea, dark epic digital painting, dramatic chiaroscuro lighting, muted monochrome palette with a single warm bronze accent #b08d57, painterly brushstrokes, seinen atmosphere --ar 4:5 --no rainbow colors, explosion, text, watermark</t>
+          <t>early 1900s battleship emerging half-real from a wall of sea fog, hull streaked with rust, gun turrets silent, no flag identifiable, the fog actively swallowing its stern as if unwriting it, cold heavy sea, dramatic chiaroscuro lighting, muted monochrome palette with a single warm bronze accent #b08d57, seinen atmosphere --no rainbow colors, explosion, text, watermark</t>
         </is>
       </c>
     </row>
@@ -4998,7 +4998,7 @@
       </c>
       <c r="S61" s="5" t="inlineStr">
         <is>
-          <t>ageless figure in layered robes from no single era standing in an impossible library where shelves curve into fog, holding an open book whose pages are blank, face half-lost in shadow beneath a deep hood, motes of golden dust orbiting like slow time, subject centered upper half, dark epic digital painting, dramatic chiaroscuro lighting, muted monochrome palette with a single warm bronze accent #b08d57, painterly brushstrokes, seinen atmosphere --ar 4:5 --no rainbow colors, wizard fantasy, text, watermark</t>
+          <t>ageless figure in layered robes from no single era standing in an impossible library where shelves curve into fog, holding an open book whose pages are blank, face half-lost in shadow beneath a deep hood, motes of golden dust orbiting like slow time, subject centered upper half, dramatic chiaroscuro lighting, muted monochrome palette with a single warm bronze accent #b08d57, seinen atmosphere --no rainbow colors, wizard fantasy, text, watermark</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: les 60 prompts réécrits en formule v5.2 (splash Riot x rétro-futur Travelers, présent 2049) ; xlsx/csv régénérés
- Chaque prompt : scène en une phrase, suit Alita carbone mat, monde
  cassette-futurism (CRT/câbles/béton/sodium) ou monde d'époque, duo de
  complémentaires + key light sujet nommée, bloc splash Riot, négatifs
  anti-fantasy
- Duos : RIKKEN bleu/ambre, KAIROS rouge/cyan, Époques bronze/or + froid
- R13 recalé (civil aspiré sans combinaison), R05 visage humain imposé,
  R14 sans créatures, full art = sujet dans les 55% hauts
- En-tête : moodboard LoL ON, stylize 200-400, régénération des 23 forgées

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/SET01-production.xlsx
+++ b/docs/SET01-production.xlsx
@@ -709,7 +709,7 @@
       </c>
       <c r="S2" s="5" t="inlineStr">
         <is>
-          <t>young female recruit in a plain matte black pre-CELL training bodysuit with small sensor pads, standing alert in a dark underground RIKKEN training hall, black metal walls with faint blue LED strips, determined tired eyes, subject centered upper half, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated blue accent #3d8fd6, seinen atmosphere --no neon everywhere, rainbow colors, iron man style, text, watermark</t>
+          <t>young female recruit in a matte black pre-CELL training bodysuit with sensor pads, standing alert in an underground RIKKEN training hall, cold blue key light from a hovering training drone on her face, warm amber target lights glowing behind her, CRT monitors and thick cables along brutalist concrete walls, retro-futuristic evangelion atmosphere, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no medieval knight armor, fantasy armor, text, watermark</t>
         </is>
       </c>
     </row>
@@ -792,7 +792,7 @@
       </c>
       <c r="S3" s="5" t="inlineStr">
         <is>
-          <t>female engineer in dark RIKKEN work uniform and cap repairing massive energy conduits deep under Odaiba, cold blue-white glow of the transfer core lighting her face from below, wrench in hand, cathedral-scale machinery, subject centered upper half, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated blue accent #3d8fd6, seinen atmosphere --no neon everywhere, rainbow colors, text, watermark</t>
+          <t>female engineer in a dark RIKKEN work uniform and cap repairing a massive energy conduit deep under odaiba, blue-white core glow lighting her face from below, warm amber work lamps and CRT gauges around her, cathedral-scale machinery and thick cables, retro-futuristic evangelion atmosphere, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no fantasy armor, text, watermark</t>
         </is>
       </c>
     </row>
@@ -877,7 +877,7 @@
       </c>
       <c r="S4" s="5" t="inlineStr">
         <is>
-          <t>female operative in a sleek black biotech suit with modular plates, thin water conduits glowing soft cyan along forearms and collar, fine mist condensing around her hands, calm ready stance in a dark concrete hall, subject centered upper half, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated cyan accent, contained light lines, seinen atmosphere --no neon everywhere, rainbow colors, iron man style, text, watermark</t>
+          <t>female operative in a sleek matte black high-tech exosuit with segmented mechanical armor plates like alita battle angel, thin water conduits glowing cyan along her forearms, fine mist condensing around her open hands, cyan key light from her own conduits on her face, warm sodium lights and thick cables in the concrete hall behind, retro-futuristic evangelion atmosphere, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no medieval knight armor, fantasy armor, ornate gold trim, text, watermark</t>
         </is>
       </c>
     </row>
@@ -960,7 +960,7 @@
       </c>
       <c r="S5" s="5" t="inlineStr">
         <is>
-          <t>female scout in a sleek dark biotech suit sprinting through a foggy 19th century parisian construction site at night, wooden scaffolding and iron beams in the mist, subtle motion blur, aerodynamic suit panels with faint blue light lines, subject centered upper half, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated blue accent #3d8fd6, seinen atmosphere --no neon everywhere, rainbow colors, eiffel tower recognizable, text, watermark</t>
+          <t>female scout in a sleek matte black high-tech exosuit with segmented armor plates like alita battle angel, faint blue glowing seams, crouched on wooden scaffolding above a foggy 19th century parisian construction site at dusk, warm amber gaslight beside her illuminating her face, violet evening sky behind the iron beams, her futuristic suit the only modern element in the era, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no eiffel tower, medieval knight armor, fantasy armor, text, watermark</t>
         </is>
       </c>
     </row>
@@ -1043,7 +1043,7 @@
       </c>
       <c r="S6" s="5" t="inlineStr">
         <is>
-          <t>massive sentinel in a heavy-plated dark biotech suit standing guard before a circular time-transfer platform, faint blue-white glow rising from the platform ring behind him, arms crossed, immovable, black metal hall with blue LED strips, subject centered upper half, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated blue accent #3d8fd6, seinen atmosphere --no neon everywhere, rainbow colors, iron man style, giant mecha, text, watermark</t>
+          <t>towering broad man in a heavy matte black segmented exosuit with thick mechanical shoulder plates, helmet off revealing a scarred stern face, arms crossed before a circular transfer platform, blue-white ring glow rising behind him, amber warning lights and thick cables on the brutalist concrete walls, retro-futuristic evangelion atmosphere, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no medieval knight armor, fantasy armor, giant robot, full helmet covering face, text, watermark</t>
         </is>
       </c>
     </row>
@@ -1126,7 +1126,7 @@
       </c>
       <c r="S7" s="5" t="inlineStr">
         <is>
-          <t>stern analyst in dark institutional uniform at a desk of translucent holographic timelines and candidate files, glasses reflecting pale blue data, dark office of the recruitment division at night, subject centered upper half, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated blue accent #3d8fd6, seinen atmosphere --no neon everywhere, rainbow colors, cyberpunk pink purple, text, watermark</t>
+          <t>stern analyst in a dark institutional uniform at a desk stacked with candidate files, round glasses reflecting pale blue light from a wall of CRT screens showing personnel records, warm amber desk lamp on his face, dark recruitment office at night with thick cables, retro-futuristic atmosphere, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no fantasy armor, cyberpunk pink purple, text, watermark</t>
         </is>
       </c>
     </row>
@@ -1201,7 +1201,7 @@
       </c>
       <c r="S8" s="5" t="inlineStr">
         <is>
-          <t>human silhouette dissolving into fine ascending blue-white light lines on a circular transfer platform, empty dark facility, the light column is the only bright source, sense of sudden departure, a dropped object still falling where the person stood, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated blue accent #3d8fd6, seinen atmosphere --no neon everywhere, rainbow colors, text, watermark</t>
+          <t>human silhouette dissolving upward into a column of blue-white light on a circular transfer platform, a dropped coffee mug still falling where the person stood, dark empty facility hall with CRT control panels and amber standby lights, the light column blazing as the only bright source, retro-futuristic evangelion atmosphere, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, atmospheric detailed background --no fantasy magic portal, text, watermark</t>
         </is>
       </c>
     </row>
@@ -1276,7 +1276,7 @@
       </c>
       <c r="S9" s="5" t="inlineStr">
         <is>
-          <t>holographic briefing table projecting layered maps of seven different historical eras, gloved hands of unseen officers pointing at a blank unmapped region, dark war-room of the RIKKEN facility, papers and cold coffee, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated blue accent #3d8fd6, seinen atmosphere --no neon everywhere, rainbow colors, text, watermark</t>
+          <t>holographic briefing table projecting layered blue maps of seven historical eras, gloved hands of unseen officers pointing at one blank unmapped region, warm amber light from scattered papers and cold coffee cups, dark war-room with CRT screens and thick cables, retro-futuristic evangelion atmosphere, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, atmospheric detailed background --no fantasy magic, text, watermark</t>
         </is>
       </c>
     </row>
@@ -1361,7 +1361,7 @@
       </c>
       <c r="S10" s="5" t="inlineStr">
         <is>
-          <t>young franco-senegalese woman medic in a sleek black biotech suit, thin cyan nano-fluid conduits glowing along her forearms, open palm with fine diffuser pores emitting soft cyan light, clinical calm expression, dark field-hospital corner of a mission camp, subject centered upper half, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated cyan accent, seinen atmosphere --no neon everywhere, rainbow colors, iron man style, text, watermark</t>
+          <t>young franco-senegalese woman medic kneeling beside a wounded soldier in a dark field hospital tent, open palm emitting soft cyan light from fine diffuser pores in her matte black segmented exosuit glove, cyan conduits glowing along her forearm, warm lantern light against the cyan glow on her calm face, green CRT medical monitors behind her, retro-futuristic atmosphere, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no medieval knight armor, fantasy armor, text, watermark</t>
         </is>
       </c>
     </row>
@@ -1446,7 +1446,7 @@
       </c>
       <c r="S11" s="5" t="inlineStr">
         <is>
-          <t>young japanese woman in a sleek dark biotech suit, fine fractal sensor lines glowing deep blue across her forearms, extended HUD visor over her eyes reflecting cascading probability data, hyper-focused expression, dark analysis chamber, subject centered upper half, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated deep blue accent, seinen atmosphere --no neon everywhere, rainbow colors, cyberpunk pink purple, text, watermark</t>
+          <t>young japanese woman in a sleek matte black high-tech exosuit with segmented armor plates like alita battle angel, wide HUD visor over her eyes reflecting cascading blue probability data, standing in a dark analysis room lit by a wall of CRT screens, deep blue key light on her face, amber standby lights and thick cables in the background, retro-futuristic evangelion atmosphere, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no medieval knight armor, fantasy armor, ornate gold trim, text, watermark</t>
         </is>
       </c>
     </row>
@@ -1513,7 +1513,7 @@
       </c>
       <c r="S12" s="5" t="inlineStr">
         <is>
-          <t>male traveler in a sleek dark biotech suit with contained ember-like combustion channels along arms and shoulders, heat shimmer rising from his gauntlets, embers drifting in a dark testing chamber, controlled and calm, no flames raging, subject centered upper half, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated ember orange-red accent, seinen atmosphere --no neon everywhere, rainbow colors, fire everywhere, iron man style, text, watermark</t>
+          <t>male traveler in a sleek matte black segmented exosuit like alita battle angel with contained ember-orange combustion channels along his arms and shoulders, heat shimmer rising from his gauntlets, embers drifting in a dark testing chamber, warm orange key light from his own conduits on his calm face, cool teal shadows and CRT monitors behind, retro-futuristic atmosphere, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no medieval knight armor, fantasy armor, fire everywhere, text, watermark</t>
         </is>
       </c>
     </row>
@@ -1596,7 +1596,7 @@
       </c>
       <c r="S13" s="5" t="inlineStr">
         <is>
-          <t>veteran escort traveler in a heavy dark biotech suit with thick worn plates and old mission scars on the armor, standing protectively in a doorway of black metal, grey temples, tired unshakable eyes, faint blue light lines, subject centered upper half, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated blue accent #3d8fd6, seinen atmosphere --no neon everywhere, rainbow colors, iron man style, text, watermark</t>
+          <t>veteran traveler with grey temples in a heavy matte black segmented exosuit with thick worn armor plates and old mission scars, standing protectively in a steel doorway, warm amber corridor light behind him, faint blue glowing seams on his suit, tired unshakable eyes lit by a cool overhead lamp, brutalist concrete and thick cables, retro-futuristic atmosphere, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no medieval knight armor, fantasy armor, ornate gold trim, text, watermark</t>
         </is>
       </c>
     </row>
@@ -1671,7 +1671,7 @@
       </c>
       <c r="S14" s="5" t="inlineStr">
         <is>
-          <t>traveler mid-dematerialization into blue-white light lines while reaching desperately toward the viewer, dark collapsed historical ruin around, dust and debris frozen mid-air, urgency and rescue, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated blue accent #3d8fd6, seinen atmosphere --no neon everywhere, rainbow colors, text, watermark</t>
+          <t>a man in 2049 civilian clothes being pulled off his feet toward a blazing column of blue-white light, one arm already dissolving into particles of light, terrified face turned toward the viewer, dark transfer chamber with CRT control panels flashing red alerts, thick cables whipping toward the column, retro-futuristic evangelion atmosphere, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no fantasy magic portal, text, watermark</t>
         </is>
       </c>
     </row>
@@ -1746,7 +1746,7 @@
       </c>
       <c r="S15" s="5" t="inlineStr">
         <is>
-          <t>translucent geometric energy dome protecting a squad of dark-suited travelers kneeling on a transfer platform, impacts flaring softly on the dome surface, dark hall beyond, the dome light is faint blue and contained, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated blue accent #3d8fd6, seinen atmosphere --no neon everywhere, rainbow colors, text, watermark</t>
+          <t>translucent blue energy dome protecting a squad of travelers in matte black segmented exosuits kneeling on a transfer platform, warm amber sparks flaring where impacts hit the dome surface, dark brutalist hall with CRT panels and cables beyond, the dome glow lighting the squad from above, retro-futuristic evangelion atmosphere, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, atmospheric detailed background --no medieval knight armor, fantasy armor, creatures, monsters, text, watermark</t>
         </is>
       </c>
     </row>
@@ -1813,7 +1813,7 @@
       </c>
       <c r="S16" s="5" t="inlineStr">
         <is>
-          <t>female squad coordinator in dark RIKKEN officer uniform standing before a wall of mission screens showing three teams in different eras, headset on, one hand raised mid-order, dark control room lit by pale blue monitors, subject centered upper half, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated blue accent #3d8fd6, seinen atmosphere --no neon everywhere, rainbow colors, text, watermark</t>
+          <t>female squad coordinator in a dark RIKKEN officer uniform standing before a wall of CRT mission screens showing three teams in three different eras, headset on, one hand raised mid-order, pale blue monitor light on her face, warm amber comm lights and thick cables around the dark control room, retro-futuristic evangelion atmosphere, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no fantasy armor, text, watermark</t>
         </is>
       </c>
     </row>
@@ -1902,7 +1902,7 @@
       </c>
       <c r="S17" s="5" t="inlineStr">
         <is>
-          <t>young russian man with insolent grin mid-parkour leap across dark rooftops, sleek black biotech suit with visible nitro thrusters on calves and back glowing warm orange, aerodynamic panels retracting, motion energy, subject centered upper half, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated warm orange accent, contained light lines, seinen atmosphere --no neon everywhere, rainbow colors, iron man style, text, watermark</t>
+          <t>young russian traveler with slicked blond hair grinning insolently, crouched low on a rooftop edge ready to launch, orange combustion glow flaring from the calf conduits of his matte black segmented exosuit like alita battle angel, orange key light from his own conduits on his face, teal-shadowed 2049 tokyo skyline with distant neon signs behind him, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no medieval knight armor, fantasy armor, fire everywhere, ornate gold trim, text, watermark</t>
         </is>
       </c>
     </row>
@@ -1987,7 +1987,7 @@
       </c>
       <c r="S18" s="5" t="inlineStr">
         <is>
-          <t>traveler in a sleek dark biotech suit standing in a foggy historical battlefield, rusted iron debris and broken blades levitating in a slow orbit around him, faint magnetic field distortion, contained pale blue light lines on his suit, subject centered upper half, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated blue accent #3d8fd6, seinen atmosphere --no neon everywhere, rainbow colors, iron man style, text, watermark</t>
+          <t>traveler in a sleek matte black segmented exosuit like alita battle angel standing in a foggy historical battlefield, rusted iron debris and broken blades levitating in a slow orbit around him, pale blue glowing seams lighting his face from below, warm bronze fog and eroded earthworks behind, his futuristic suit the only modern element in the era, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no medieval knight armor, fantasy armor, fantasy magic, text, watermark</t>
         </is>
       </c>
     </row>
@@ -2062,7 +2062,7 @@
       </c>
       <c r="S19" s="5" t="inlineStr">
         <is>
-          <t>the massive spherical energy core of the RIKKEN central deep under Odaiba surging with blue-white power, catwalks and tiny engineer silhouettes dwarfed by the machine, conduits blazing with contained light, industrial cathedral scale, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated blue accent #3d8fd6, seinen atmosphere --no neon everywhere, rainbow colors, explosion, text, watermark</t>
+          <t>colossal underground transfer core beneath tokyo blazing with blue-white overload, tiny engineers running on steel gantries silhouetted against the light, cathedral-scale machinery with thick cables and amber warning strobes, steam venting from brutalist concrete walls, retro-futuristic evangelion industrial atmosphere, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, atmospheric detailed background --no fantasy magic, spaceship, explosion, text, watermark</t>
         </is>
       </c>
     </row>
@@ -2129,7 +2129,7 @@
       </c>
       <c r="S20" s="5" t="inlineStr">
         <is>
-          <t>stern japanese woman in her fifties in an impeccable dark RIKKEN uniform, seated alone at an elevated jury desk in the white immaculate test center, arms crossed, evaluating gaze cutting downward at the viewer, clinical white light, one blue insignia, subject centered upper half, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated blue accent #3d8fd6, seinen atmosphere --no neon everywhere, rainbow colors, text, watermark</t>
+          <t>stern japanese woman in her fifties in an impeccable dark RIKKEN uniform seated at an elevated jury desk in a white immaculate test center, evaluating gaze cutting down at the viewer, cold clinical white key light on her face, one glowing blue insignia on her collar, warm amber file lamps on the desk, subject in the upper half of the frame, lower third calm and atmospheric, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no fantasy armor, text, watermark</t>
         </is>
       </c>
     </row>
@@ -2218,7 +2218,7 @@
       </c>
       <c r="S21" s="5" t="inlineStr">
         <is>
-          <t>imposing japanese man in his sixties, granite face and grey brush cut, wearing a first-generation biotech suit with visible patinated copper and brass conductors, thick old-school plates, mechanical piston joints, standing like a rock in a dark hangar, quiet overwhelming aura, subject centered upper half, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated warm brass accent, seinen atmosphere --no neon everywhere, rainbow colors, iron man style, text, watermark</t>
+          <t>imposing japanese man in his sixties with a granite face and grey brush cut wearing a first-generation exosuit with patinated copper conductors, thick old-school plates and mechanical piston joints, standing like a rock in a dark hangar, warm brass key light from his suit's aged conductors on his face, cool blue hangar lights and thick cables behind, subject in the upper half of the frame, lower third atmospheric, retro-futuristic atmosphere, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no medieval knight armor, fantasy armor, ornate gold trim, text, watermark</t>
         </is>
       </c>
     </row>
@@ -2285,7 +2285,7 @@
       </c>
       <c r="S22" s="5" t="inlineStr">
         <is>
-          <t>broad-shouldered chinese man in a heavy dark biotech suit, forearm and chest plates condensing into matte-black liquid-stone density, one massive fist wrapped in a compressive distortion aura, cracked concrete under his feet, dark testing arena, subject centered upper half, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated blue accent #3d8fd6, seinen atmosphere --no neon everywhere, rainbow colors, hulk, giant mecha, text, watermark</t>
+          <t>broad-shouldered chinese man in a heavy matte black segmented exosuit like alita battle angel, forearm and chest plates condensed into liquid-stone density, one massive fist wrapped in a subtle compressive distortion, cracked concrete radiating under his feet in a dark testing arena, blue key light from arena floodlights on his face, warm dust haze behind, subject in the upper half of the frame, lower third atmospheric, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no medieval knight armor, fantasy armor, hulk, giant robot, text, watermark</t>
         </is>
       </c>
     </row>
@@ -2374,7 +2374,7 @@
       </c>
       <c r="S23" s="5" t="inlineStr">
         <is>
-          <t>19 year old slim french-japanese young man, light beige tousled hair with dark strands and one single vivid red strand over his right brow, thin scar on right cheekbone, grey almond eyes, wearing a sleek black prototype biotech suit with modular reconfiguring panels, a small engraved golden circle glowing softly on his chest, faint multi-hued light lines syncing along his arms, dark platform hall, subject centered upper half, dramatic chiaroscuro lighting, muted monochrome palette with red strand and golden circle as only accents, seinen atmosphere --no neon everywhere, rainbow colors, iron man style, text, watermark</t>
+          <t>19 year old slim french-japanese young man with light beige tousled hair, one single vivid red strand over his right brow and a thin scar on his right cheekbone, standing at the center of a transfer platform in a sleek matte black prototype exosuit with modular reconfiguring panels, a small engraved golden circle glowing on his chest, blue-white light column rising behind him, blue key light on his determined face, CRT monitors and thick cables around the platform ring, subject in the upper half of the frame, lower third atmospheric, retro-futuristic evangelion atmosphere, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no medieval knight armor, fantasy armor, ornate gold trim, text, watermark</t>
         </is>
       </c>
     </row>
@@ -2457,7 +2457,7 @@
       </c>
       <c r="S24" s="5" t="inlineStr">
         <is>
-          <t>unremarkable middle-aged agent in a dark RIKKEN staff uniform standing in a facility corridor at 3am, authentic institute badge on his chest, half of his face swallowed by shadow, the other half perfectly ordinary, one tiny red LED reflected in his eye, subject centered upper half, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated red accent #c23b4e, seinen atmosphere --no neon everywhere, rainbow colors, text, watermark</t>
+          <t>unremarkable middle-aged agent in a dark RIKKEN staff uniform standing in a facility corridor at 3am, authentic institute badge on his chest, half his face in shadow, one tiny red LED reflected in his eye, cold blue corridor light and a distant red security light down the hall, CRT panels and thick cables on the walls, retro-futuristic blade runner atmosphere, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no fantasy armor, text, watermark</t>
         </is>
       </c>
     </row>
@@ -2524,7 +2524,7 @@
       </c>
       <c r="S25" s="5" t="inlineStr">
         <is>
-          <t>young candidate in recruit fatigues standing in line at the white RIKKEN test center, posture identical to the others but eyes measuring the room like a professional, faint red thread bracelet under his sleeve, clinical white light, half his face in shadow, subject centered upper half, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated red accent #c23b4e, seinen atmosphere --no neon everywhere, rainbow colors, text, watermark</t>
+          <t>young candidate in recruit fatigues standing in line at the white RIKKEN test center, posture identical to the others but eyes measuring the room like a professional, thin red thread bracelet under his sleeve, cold clinical white key light, other candidates softly blurred around him, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no fantasy armor, text, watermark</t>
         </is>
       </c>
     </row>
@@ -2591,7 +2591,7 @@
       </c>
       <c r="S26" s="5" t="inlineStr">
         <is>
-          <t>operative in a stolen dark biotech suit moving silently through an empty facility corridor at night, suit light lines flickering red and miscalibrated, one hand trailing along the wall, security camera dead behind him, subject centered upper half, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated red accent #c23b4e, contained light lines, seinen atmosphere --no neon everywhere, rainbow colors, iron man style, text, watermark</t>
+          <t>operative in a stolen matte black segmented exosuit moving silently through an empty facility corridor at night, suit seams flickering red and miscalibrated, one hand trailing along the wall, a dead security camera behind him, cold blue emergency lighting with his red seams as the warm counterpoint, brutalist concrete and cables, retro-futuristic blade runner atmosphere, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no medieval knight armor, fantasy armor, text, watermark</t>
         </is>
       </c>
     </row>
@@ -2658,7 +2658,7 @@
       </c>
       <c r="S27" s="5" t="inlineStr">
         <is>
-          <t>watcher in dark civilian clothes standing on a rooftop overlooking Tokyo bay at night, binoculars lowered, patient posture, the city lights muted and grey except one distant red aircraft beacon, wind in his coat, subject centered upper half, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated red accent #c23b4e, seinen atmosphere --no neon everywhere, rainbow colors, cyberpunk, text, watermark</t>
+          <t>patient watcher in dark 2049 civilian clothes standing on a rooftop overlooking tokyo bay at night, binoculars lowered, wind in his coat, the city lights muted and grey except one distant red aircraft beacon, cool blue night key light on his face with the red beacon reflected in his eyes, retro-futuristic blade runner atmosphere, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no fantasy armor, cyberpunk pink purple overload, text, watermark</t>
         </is>
       </c>
     </row>
@@ -2741,7 +2741,7 @@
       </c>
       <c r="S28" s="5" t="inlineStr">
         <is>
-          <t>kairos fighter in a mismatched stolen biotech suit, panels from different CELL generations bolted together, red light lines sputtering and glitching at the seams, aggressive hunched stance in a dark parking structure, subject centered upper half, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated red accent #c23b4e, seinen atmosphere --no neon everywhere, rainbow colors, iron man style, text, watermark</t>
+          <t>kairos fighter in a mismatched stolen exosuit with segmented panels from different CELL generations bolted together, red seams sputtering and glitching, aggressive hunched stance in a dark parking structure, red key light from his own faulty conduits on his face, warm sodium lights and thick pillars behind, retro-futuristic blade runner atmosphere, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no medieval knight armor, fantasy armor, text, watermark</t>
         </is>
       </c>
     </row>
@@ -2808,7 +2808,7 @@
       </c>
       <c r="S29" s="5" t="inlineStr">
         <is>
-          <t>cold professional woman in a tailored dark coat standing over an open briefcase of precise tech instruments, surgical calm, dark hotel room with Tokyo night skyline muted behind glass, one red instrument light, subject centered upper half, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated red accent #c23b4e, seinen atmosphere --no neon everywhere, rainbow colors, blood, text, watermark</t>
+          <t>cold professional woman in a tailored dark coat standing over an open briefcase of precise tech instruments, surgical calm, dark hotel room with the muted tokyo night skyline behind glass, one red instrument light on her face against cool blue window light, retro-futuristic blade runner atmosphere, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no fantasy armor, blood, text, watermark</t>
         </is>
       </c>
     </row>
@@ -2875,7 +2875,7 @@
       </c>
       <c r="S30" s="5" t="inlineStr">
         <is>
-          <t>executive in an impeccable suit standing in a glass corner office above Tokyo at night, back to the viewer, reflection in the window showing a face we cannot quite read, red seal stamp resting on signed documents, subject centered upper half, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated red accent #c23b4e, seinen atmosphere --no neon everywhere, rainbow colors, text, watermark</t>
+          <t>executive in an impeccable suit standing in a glass corner office above tokyo at night, back to the viewer, his unreadable face reflected in the window, red seal stamp resting on signed documents, warm desk lamp against the cool blue city glow, retro-futuristic blade runner atmosphere, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no fantasy armor, text, watermark</t>
         </is>
       </c>
     </row>
@@ -2942,7 +2942,7 @@
       </c>
       <c r="S31" s="5" t="inlineStr">
         <is>
-          <t>close-up of a gloved hand sliding a thin red-sealed dossier across a polished dark table toward a trembling bare hand, tea untouched, faces out of frame, dark meeting room, the seal is the only color, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated red accent #c23b4e, seinen atmosphere --no neon everywhere, rainbow colors, text, watermark</t>
+          <t>close-up of a gloved hand sliding a thin red-sealed dossier across a polished dark table toward a trembling bare hand, tea untouched, faces out of frame, warm lamp light pooling on the table with the red seal as the sharpest color, dark meeting room with a CRT glowing in the background, retro-futuristic atmosphere, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the hands, atmospheric detailed background --no fantasy magic, text, watermark</t>
         </is>
       </c>
     </row>
@@ -3009,7 +3009,7 @@
       </c>
       <c r="S32" s="5" t="inlineStr">
         <is>
-          <t>circular time-transfer platform short-circuiting in a dark hall, its blue ring guttering out while thin red warning strobes sweep the walls, sparks raining, a small sabotage device blinking red at the platform base, no people, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated red accent #c23b4e, seinen atmosphere --no neon everywhere, rainbow colors, explosion, text, watermark</t>
+          <t>circular transfer platform short-circuiting in a dark hall, its blue ring guttering out while red warning strobes sweep the walls, sparks raining from severed thick cables, a small sabotage device blinking red at the platform base, no people, CRT panels flashing errors, retro-futuristic evangelion atmosphere, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, atmospheric detailed background --no fantasy magic, explosion, text, watermark</t>
         </is>
       </c>
     </row>
@@ -3076,7 +3076,7 @@
       </c>
       <c r="S33" s="5" t="inlineStr">
         <is>
-          <t>female kairos operative in a dark tech coat raising a small parasite emitter, translucent red interference waves rippling from it, a distant traveler's suit light lines visibly stuttering and dying, dark facility hall, subject centered upper half, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated red accent #c23b4e, seinen atmosphere --no neon everywhere, rainbow colors, text, watermark</t>
+          <t>female kairos operative in a dark tech coat over a matte black segmented exosuit raising a small parasite emitter, translucent red interference waves rippling from it, a distant traveler's blue suit seams visibly stuttering and dying, red key light from the emitter on her focused face, dark facility hall with cables and CRT panels, retro-futuristic blade runner atmosphere, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no medieval knight armor, fantasy armor, text, watermark</t>
         </is>
       </c>
     </row>
@@ -3143,7 +3143,7 @@
       </c>
       <c r="S34" s="5" t="inlineStr">
         <is>
-          <t>lean duelist in a stolen sleek biotech suit, contained electric arcs crawling between his gauntlets, red-tinged capacitor lines pulsing unstably along his spine, combat stance in a rain-slick dark alley, subject centered upper half, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated red accent #c23b4e, seinen atmosphere --no neon everywhere, rainbow colors, lightning storm, iron man style, text, watermark</t>
+          <t>lean duelist in a stolen matte black segmented exosuit like alita battle angel, contained electric arcs crawling between his gauntlets, red-tinged capacitor seams pulsing along his spine, combat stance in a rain-slick dark alley, white-blue arc light on his face against the red seams, cyan reflections in the puddles, retro-futuristic blade runner atmosphere, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no medieval knight armor, fantasy armor, lightning storm, text, watermark</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3210,7 @@
       </c>
       <c r="S35" s="5" t="inlineStr">
         <is>
-          <t>charming recruiter in RIKKEN colors leaning across an interview table toward an unseen candidate, warm practiced smile that stops below the eyes, red pen turning slowly between his fingers, dark interview room, subject centered upper half, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated red accent #c23b4e, seinen atmosphere --no neon everywhere, rainbow colors, text, watermark</t>
+          <t>charming recruiter in RIKKEN colors leaning across an interview table toward an unseen candidate, warm practiced smile that stops below the eyes, red pen turning slowly between his fingers, warm desk lamp on his face against the cool dark interview room, a CRT recorder blinking in the corner, retro-futuristic atmosphere, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no fantasy armor, text, watermark</t>
         </is>
       </c>
     </row>
@@ -3277,7 +3277,7 @@
       </c>
       <c r="S36" s="5" t="inlineStr">
         <is>
-          <t>huge enforcer in a reinforced dark suit filling a narrow basement corridor of the facility, head bowed under the ceiling, knuckles wrapped in red-lit compression bands, pipes and steam around him, subject centered upper half, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated red accent #c23b4e, seinen atmosphere --no neon everywhere, rainbow colors, hulk, giant mecha, text, watermark</t>
+          <t>huge enforcer in a reinforced matte black segmented exosuit filling a narrow basement corridor, head bowed under the ceiling, knuckles wrapped in red-lit compression bands, steam from pipes catching the red glow, warm sodium light behind him and cold shadows ahead, brutalist concrete and thick cables, retro-futuristic atmosphere, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no medieval knight armor, fantasy armor, hulk, giant robot, text, watermark</t>
         </is>
       </c>
     </row>
@@ -3344,7 +3344,7 @@
       </c>
       <c r="S37" s="5" t="inlineStr">
         <is>
-          <t>a traveler's biotech suit mid-activation abruptly failing, its blue light lines shattering into static as a translucent red interference wave passes through the frame, the traveler's silhouette frozen mid-gesture in a dark hall, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated red accent #c23b4e, seinen atmosphere --no neon everywhere, rainbow colors, text, watermark</t>
+          <t>a traveler's matte black exosuit mid-activation abruptly failing, its blue glowing seams shattering into static as a translucent red interference wave passes through the frame, the traveler's silhouette frozen mid-gesture in a dark hall, blue light dying into red across the scene, CRT panels glitching behind, retro-futuristic evangelion atmosphere, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, atmospheric detailed background --no fantasy magic, text, watermark</t>
         </is>
       </c>
     </row>
@@ -3411,7 +3411,7 @@
       </c>
       <c r="S38" s="5" t="inlineStr">
         <is>
-          <t>human figure being torn backward out of a historical scene into red-black static, the scene itself continuing undisturbed around the void he leaves, fingers clawing at air, sense of violent temporal removal, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated red accent #c23b4e, seinen atmosphere --no neon everywhere, rainbow colors, gore, text, watermark</t>
+          <t>human figure being torn backward out of a warm historical street scene into red-black static, fingers clawing at air, the era continuing undisturbed around the void he leaves, warm bronze daylight in the scene against the cold red-black tear, sense of violent temporal removal, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no fantasy magic portal, gore, text, watermark</t>
         </is>
       </c>
     </row>
@@ -3478,7 +3478,7 @@
       </c>
       <c r="S39" s="5" t="inlineStr">
         <is>
-          <t>female kairos agent in a stolen suit kneeling in a foggy blind-zone battlefield, prying a relic from the mud into a red-lit containment case, disturbed historical dead around her under the mist, disrespectful haste, subject centered upper half, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated red accent #c23b4e, seinen atmosphere --no neon everywhere, rainbow colors, gore, text, watermark</t>
+          <t>female kairos agent in a stolen matte black segmented exosuit kneeling in a foggy blind-zone battlefield, prying a relic from the mud into a red-lit containment case, red case light on her hurried face against the warm bronze fog of the era, disturbed ancient earth around her, her modern suit profane against the historical dead ground, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no medieval knight armor, fantasy armor, gore, skeletons, text, watermark</t>
         </is>
       </c>
     </row>
@@ -3545,7 +3545,7 @@
       </c>
       <c r="S40" s="5" t="inlineStr">
         <is>
-          <t>interrogator in an immaculate dark uniform standing beside an empty steel chair in a blinding white interrogation room, one red recording light on the wall, his shadow falling across the chair, quiet menace, subject centered upper half, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated red accent #c23b4e, seinen atmosphere --no neon everywhere, rainbow colors, text, watermark</t>
+          <t>interrogator in an immaculate dark uniform standing beside an empty steel chair in a blinding white interrogation room, his long shadow falling across the chair, one red recording light on the wall reflected in his glasses, cold white key light with the red light as the only color, quiet menace, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no fantasy armor, text, watermark</t>
         </is>
       </c>
     </row>
@@ -3612,7 +3612,7 @@
       </c>
       <c r="S41" s="5" t="inlineStr">
         <is>
-          <t>kairos operative in a sleek stolen biotech suit standing calmly while a swarm of palm-sized drones orbits him in a slow red-lit constellation, each drone eye a tiny red point, dark server hall, subject centered upper half, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated red accent #c23b4e, contained light lines, seinen atmosphere --no neon everywhere, rainbow colors, iron man style, text, watermark</t>
+          <t>kairos operative in a sleek stolen matte black segmented exosuit standing calmly while a swarm of palm-sized drones orbits him in a slow constellation, each drone eye a tiny red point, red drone lights rimming his silhouette against the cool blue glow of a dark server hall, thick cables and blinking racks behind, retro-futuristic blade runner atmosphere, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no medieval knight armor, fantasy armor, text, watermark</t>
         </is>
       </c>
     </row>
@@ -3679,7 +3679,7 @@
       </c>
       <c r="S42" s="5" t="inlineStr">
         <is>
-          <t>monumental cracked clock face suspended in darkness, thin red light bleeding through the fracture lines, a single silhouette stepping through the largest crack as through a door, shards of time frozen around, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated red accent #c23b4e, seinen atmosphere --no neon everywhere, rainbow colors, text, watermark</t>
+          <t>monumental cracked clock face suspended in darkness, thin red light bleeding through the fracture lines, a single silhouette stepping through the largest crack as through a door, cold grey clockwork detail against the red glow, subject in the upper half of the frame, lower third dark and atmospheric, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, atmospheric detailed background --no fantasy magic portal, text, watermark</t>
         </is>
       </c>
     </row>
@@ -3762,7 +3762,7 @@
       </c>
       <c r="S43" s="5" t="inlineStr">
         <is>
-          <t>distinguished japanese director in his fifties in a flawless dark suit, seated at a directorial desk high above Tokyo night, hands calmly folded, wearing a warm gentle smile that is slightly too perfect to be true, red seal ring on his finger, soft office light, subject centered upper half, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated red accent #c23b4e, seinen atmosphere --no neon everywhere, rainbow colors, villain sneer, text, watermark</t>
+          <t>distinguished japanese director in his fifties in a flawless dark suit seated at a directorial desk high above the tokyo night, hands calmly folded, warm gentle smile slightly too perfect to be true, warm desk lamp key light on his face, red seal ring catching the light, cool blue city glow through the glass behind him, subject in the upper half of the frame, lower third atmospheric, retro-futuristic blade runner atmosphere, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no fantasy armor, villain sneer, text, watermark</t>
         </is>
       </c>
     </row>
@@ -3829,7 +3829,7 @@
       </c>
       <c r="S44" s="5" t="inlineStr">
         <is>
-          <t>austere woman in a dark tailored suit standing in a shadowed archive of ledgers and red-stamped files, holding a single page up to a thin blade of light, faces of debtors pinned on threads behind her like a silent web, subject centered upper half, dramatic chiaroscuro lighting, muted monochrome palette with a single saturated red accent #c23b4e, seinen atmosphere --no neon everywhere, rainbow colors, text, watermark</t>
+          <t>austere woman in a dark tailored suit standing in a shadowed archive of ledgers and red-stamped files, holding a single page up into a thin blade of warm light, faces of debtors pinned on threads behind her like a silent web, warm amber blade of light on her face against the cold dark stacks, red stamps as the sharpest color, subject in the upper half of the frame, lower third atmospheric, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no fantasy armor, text, watermark</t>
         </is>
       </c>
     </row>
@@ -3918,7 +3918,7 @@
       </c>
       <c r="S45" s="5" t="inlineStr">
         <is>
-          <t>gaunt japanese man with hollow calm eyes in a matte black biotech suit, thin prismatic conductor panels shimmering faintly across shoulders and forearms, twin adaptive blades half-extended from his forearms catching a red emergency light, empty facility hall at night, subject centered upper half, dramatic chiaroscuro lighting, muted monochrome palette with prismatic shimmer and single red accent #c23b4e, seinen atmosphere --no neon everywhere, rainbow colors everywhere, iron man style, text, watermark</t>
+          <t>tall gaunt japanese man with hollow calm eyes in a long black coat over a matte black segmented exosuit, standing in falling snow at night, one raised hand crushing a glowing blue CELL core that dies between his fingers, red glowing seams under the coat, sodium street lights and a flickering CRT billboard behind, brutalist government building in the snow haze, subject in the upper half of the frame, lower third atmospheric, retro-futuristic blade runner atmosphere, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no medieval knight armor, fantasy armor, cape flowing dramatically, text, watermark</t>
         </is>
       </c>
     </row>
@@ -3985,7 +3985,7 @@
       </c>
       <c r="S46" s="5" t="inlineStr">
         <is>
-          <t>street kid in patched wool clothes and oversized cap standing in a fog-drowned parisian alley in 1888, iron scaffolding of a construction site looming as vague shapes in the mist behind, sharp knowing eyes, bronze sepia tones, the fog erasing every landmark, subject centered upper half, dramatic chiaroscuro lighting, muted monochrome palette with a single warm bronze accent #b08d57, seinen atmosphere --no eiffel tower recognizable, rainbow colors, text, watermark</t>
+          <t>street kid in patched wool clothes and an oversized cap standing in a fog-drowned parisian alley in 1888, sharp knowing eyes, warm gaslight from a lantern above him against the cool teal fog, iron scaffolding as vague shapes in the mist erasing every landmark, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no eiffel tower, modern elements, text, watermark</t>
         </is>
       </c>
     </row>
@@ -4052,7 +4052,7 @@
       </c>
       <c r="S47" s="5" t="inlineStr">
         <is>
-          <t>laundress in rough 19th century workclothes wringing linen at a river bank at dawn, thick fog hiding the far shore and every monument, her breath visible, strong tired hands, warm bronze light through the mist, subject centered upper half, dramatic chiaroscuro lighting, muted monochrome palette with a single warm bronze accent #b08d57, seinen atmosphere --no recognizable landmarks, rainbow colors, text, watermark</t>
+          <t>laundress in rough 19th century workclothes wringing linen at a river bank at dawn, strong tired hands, her breath visible, warm bronze dawn light on her face through the thick fog that hides the far shore and every monument, cold blue-grey water, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no recognizable landmarks, modern elements, text, watermark</t>
         </is>
       </c>
     </row>
@@ -4127,7 +4127,7 @@
       </c>
       <c r="S48" s="5" t="inlineStr">
         <is>
-          <t>masterless samurai in worn dark travel clothes standing at the foot of a wooden bridge swallowed by river mist, hand resting on a chipped saya, the far end of the bridge invisible, no banners no crest, flood-heavy river below, subject centered upper half, dramatic chiaroscuro lighting, muted monochrome palette with a single warm bronze accent #b08d57, seinen atmosphere --no famous castle, rainbow colors, text, watermark</t>
+          <t>masterless samurai in worn dark travel clothes standing at the foot of a wooden bridge swallowed by river mist, hand resting on a chipped saya, warm lantern light from a post beside him against the cold teal mist, the far end of the bridge invisible, no banners no crest, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no famous castle, modern elements, text, watermark</t>
         </is>
       </c>
     </row>
@@ -4194,7 +4194,7 @@
       </c>
       <c r="S49" s="5" t="inlineStr">
         <is>
-          <t>weathered stonemason in medieval work clothes laying stones of a small unfinished mountain chapel as snow begins to bury the pass, wooden scaffold creaking in the wind, mallet in cracked hands, whiteout erasing the valley below, subject centered upper half, dramatic chiaroscuro lighting, muted monochrome palette with a single warm bronze accent #b08d57, seinen atmosphere --no recognizable cathedral, rainbow colors, text, watermark</t>
+          <t>weathered stonemason in medieval work clothes laying stones of a small unfinished mountain chapel as snow buries the pass, mallet in cracked hands, warm firelight from a brazier beside him against the blue whiteout erasing the valley below, creaking wooden scaffold, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no recognizable cathedral, modern elements, text, watermark</t>
         </is>
       </c>
     </row>
@@ -4261,7 +4261,7 @@
       </c>
       <c r="S50" s="5" t="inlineStr">
         <is>
-          <t>lone roman legionary in mud-caked worn armor standing in a dark primeval forest, shield split, fog between colossal trees swallowing the rest of his column, no standard visible, exhausted defiance, moss and rain, subject centered upper half, dramatic chiaroscuro lighting, muted monochrome palette with a single warm bronze accent #b08d57, seinen atmosphere --no roman monument, rainbow colors, text, watermark</t>
+          <t>lone roman legionary in mud-caked worn armor standing in a dark primeval forest, shield split, exhausted defiance on his rain-streaked face, pale bronze light breaking through colossal trees while fog swallows the rest of his column, moss green shadows, no standard visible, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no roman monument, modern elements, fantasy armor, text, watermark</t>
         </is>
       </c>
     </row>
@@ -4328,7 +4328,7 @@
       </c>
       <c r="S51" s="5" t="inlineStr">
         <is>
-          <t>harpooner in heavy oilskins standing at the icy bow of a whaling boat locked in pack ice, harpoon planted, breath steaming, the sea and sky fused into one grey fog wall, frost in his beard, subject centered upper half, dramatic chiaroscuro lighting, muted monochrome palette with a single warm bronze accent #b08d57, seinen atmosphere --no rainbow colors, text, watermark</t>
+          <t>harpooner in heavy oilskins standing at the icy bow of a whaling boat locked in pack ice, harpoon planted, frost in his beard, warm oil lamp light on his face against the vast teal ice and the grey fog wall where sea and sky fuse, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no modern ships, text, watermark</t>
         </is>
       </c>
     </row>
@@ -4395,7 +4395,7 @@
       </c>
       <c r="S52" s="5" t="inlineStr">
         <is>
-          <t>colossal prehistoric steppe bear rearing in a blizzard on an endless white plain, fur crusted with ice, breath like smoke, its shape half-dissolved by the snowstorm that erases the horizon, primal and indifferent, subject centered upper half, dramatic chiaroscuro lighting, muted monochrome palette with a single warm bronze accent #b08d57, seinen atmosphere --no rainbow colors, text, watermark</t>
+          <t>colossal prehistoric steppe bear rearing in a blizzard on an endless white plain, fur crusted with ice, breath like smoke, pale gold dawn light catching its silhouette against the blue snowstorm that erases the horizon, primal and indifferent, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no modern elements, text, watermark</t>
         </is>
       </c>
     </row>
@@ -4462,7 +4462,7 @@
       </c>
       <c r="S53" s="5" t="inlineStr">
         <is>
-          <t>a bare human hand dissolving into drifting golden dust motes inside a single blade of late afternoon light, dark empty barn interior, the dust rising and scattering like memory, quiet and sad, dramatic chiaroscuro lighting, muted monochrome palette with a single warm bronze accent #b08d57, seinen atmosphere --no rainbow colors, skeleton, text, watermark</t>
+          <t>a bare human hand dissolving into drifting golden dust motes inside a single blade of late afternoon light, dark empty barn interior, the dust rising and scattering like memory, warm gold light against deep brown shadows, quiet and sad, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, atmospheric detailed background --no skeleton, gore, text, watermark</t>
         </is>
       </c>
     </row>
@@ -4529,7 +4529,7 @@
       </c>
       <c r="S54" s="5" t="inlineStr">
         <is>
-          <t>crowded blurry historical tavern scene, every figure slightly smeared except one perfectly sharp empty chair at the center table with a still-steaming cup before it, the absence louder than the crowd, dramatic chiaroscuro lighting, muted monochrome palette with a single warm bronze accent #b08d57, seinen atmosphere --no rainbow colors, text, watermark</t>
+          <t>crowded historical tavern scene with every figure softly blurred except one perfectly sharp empty chair at the center table, a still-steaming cup before it, warm hearth light pooling on the empty seat against the cool blurred crowd, the absence louder than the noise, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, atmospheric detailed background --no modern elements, text, watermark</t>
         </is>
       </c>
     </row>
@@ -4596,7 +4596,7 @@
       </c>
       <c r="S55" s="5" t="inlineStr">
         <is>
-          <t>barefoot young messenger girl sprinting through a narrow ancient market street before dawn, sealed letter clutched to her chest, dust rising behind her bare heels, awnings and shadows blurring past, no era landmark visible, subject centered upper half, dramatic chiaroscuro lighting, muted monochrome palette with a single warm bronze accent #b08d57, seinen atmosphere --no rainbow colors, text, watermark</t>
+          <t>barefoot young messenger girl sprinting through a narrow ancient market street before dawn, sealed letter clutched to her chest, dust rising behind her heels, warm lantern glows in the awnings against the violet pre-dawn sky, no era landmark visible, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no modern elements, text, watermark</t>
         </is>
       </c>
     </row>
@@ -4663,7 +4663,7 @@
       </c>
       <c r="S56" s="5" t="inlineStr">
         <is>
-          <t>old griot storyteller mid-tale at a night fire, hands spread wide casting long shadows, circle of captivated listeners leaning in from the darkness, sparks rising like his words, no monument no writing anywhere, subject centered upper half, dramatic chiaroscuro lighting, muted monochrome palette with a single warm bronze accent #b08d57, seinen atmosphere --no rainbow colors, text, watermark</t>
+          <t>old griot storyteller mid-tale at a night fire, hands spread wide casting long shadows, sparks rising like his words, warm fire light on his animated face against the deep blue night, circle of captivated listeners leaning in from the darkness, no monument no writing anywhere, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no modern elements, text, watermark</t>
         </is>
       </c>
     </row>
@@ -4730,7 +4730,7 @@
       </c>
       <c r="S57" s="5" t="inlineStr">
         <is>
-          <t>mountain woman warrior in furs and iron standing alone in a snowstorm at a narrow alpine pass, long spear planted, the path behind her vanishing into whiteout, ice in her braids, immovable calm, subject centered upper half, dramatic chiaroscuro lighting, muted monochrome palette with a single warm bronze accent #b08d57, seinen atmosphere --no rainbow colors, fantasy armor, text, watermark</t>
+          <t>mountain woman warrior in furs and iron standing alone in a snowstorm at a narrow alpine pass, long spear planted, ice in her braids, immovable calm, warm bronze light from a watch fire beside her against the blue whiteout that erases the path behind, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no fantasy armor, ornate gold trim, modern elements, text, watermark</t>
         </is>
       </c>
     </row>
@@ -4797,7 +4797,7 @@
       </c>
       <c r="S58" s="5" t="inlineStr">
         <is>
-          <t>wide historical landscape whose center is simply unwritten, a soft blank void swallowing the middle of the scene, the world fraying into nothing at its edges, birds flying around the absence, eerie and calm, dramatic chiaroscuro lighting, muted monochrome palette with a single warm bronze accent #b08d57, seinen atmosphere --no rainbow colors, portal, text, watermark</t>
+          <t>wide historical landscape whose center is simply unwritten, a soft pale void swallowing the middle of the scene, the world fraying into nothing at its edges, birds flying around the absence, warm bronze countryside against the cold blank void, eerie and calm, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, atmospheric detailed background --no fantasy magic portal, modern elements, text, watermark</t>
         </is>
       </c>
     </row>
@@ -4864,7 +4864,7 @@
       </c>
       <c r="S59" s="5" t="inlineStr">
         <is>
-          <t>lean swordsman in dark simple garb waiting at the far end of a mist-drowned wooden bridge, blade still sheathed, one hand raised in silent invitation, river fog erasing everything beyond ten paces, coiled stillness, subject centered upper half, dramatic chiaroscuro lighting, muted monochrome palette with a single warm bronze accent #b08d57, seinen atmosphere --no famous landmark, rainbow colors, text, watermark</t>
+          <t>lean swordsman in dark simple garb waiting at the far end of a mist-drowned wooden bridge, blade still sheathed, one hand raised in silent invitation, coiled stillness, cold steel-blue mist with a warm paper lantern glow at his feet, the river fog erasing everything beyond ten paces, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no famous landmark, modern elements, text, watermark</t>
         </is>
       </c>
     </row>
@@ -4931,7 +4931,7 @@
       </c>
       <c r="S60" s="5" t="inlineStr">
         <is>
-          <t>early 1900s battleship emerging half-real from a wall of sea fog, hull streaked with rust, gun turrets silent, no flag identifiable, the fog actively swallowing its stern as if unwriting it, cold heavy sea, dramatic chiaroscuro lighting, muted monochrome palette with a single warm bronze accent #b08d57, seinen atmosphere --no rainbow colors, explosion, text, watermark</t>
+          <t>early 1900s battleship emerging half-real from a wall of sea fog, hull streaked with rust, gun turrets silent, no flag identifiable, warm rust and bronze tones of the hull against the cold teal fog actively swallowing its stern as if unwriting it, heavy dark sea, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, atmospheric detailed background --no modern warships, explosion, text, watermark</t>
         </is>
       </c>
     </row>
@@ -4998,7 +4998,7 @@
       </c>
       <c r="S61" s="5" t="inlineStr">
         <is>
-          <t>ageless figure in layered robes from no single era standing in an impossible library where shelves curve into fog, holding an open book whose pages are blank, face half-lost in shadow beneath a deep hood, motes of golden dust orbiting like slow time, subject centered upper half, dramatic chiaroscuro lighting, muted monochrome palette with a single warm bronze accent #b08d57, seinen atmosphere --no rainbow colors, wizard fantasy, text, watermark</t>
+          <t>ageless figure in layered robes from no single era standing in an impossible library where shelves curve into fog, holding an open book whose pages are blank, face half-lost in shadow beneath a deep hood, warm golden dust motes orbiting like slow time against the cold violet fog between the shelves, subject in the upper half of the frame, lower third atmospheric, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no wizard fantasy, glowing runes, modern elements, text, watermark</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: prompts v6 — courts (~50 mots), un mouvement par image, décors tous distincts, compositions signature pour les raretés hautes ; xlsx/csv régénérés
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/SET01-production.xlsx
+++ b/docs/SET01-production.xlsx
@@ -709,7 +709,7 @@
       </c>
       <c r="S2" s="5" t="inlineStr">
         <is>
-          <t>young female recruit in a matte black pre-CELL training bodysuit with sensor pads, standing alert in an underground RIKKEN training hall, cold blue key light from a hovering training drone on her face, warm amber target lights glowing behind her, CRT monitors and thick cables along brutalist concrete walls, retro-futuristic evangelion atmosphere, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no medieval knight armor, fantasy armor, text, watermark</t>
+          <t>young female recruit in a matte black training bodysuit vaulting over an obstacle wall, morning light shafts through high skylights, dust motes, instructors watching from a gantry, blue and amber training lights, league of legends splash art, highly detailed, dynamic composition, cinematic lighting --no fantasy armor, text, watermark</t>
         </is>
       </c>
     </row>
@@ -792,7 +792,7 @@
       </c>
       <c r="S3" s="5" t="inlineStr">
         <is>
-          <t>female engineer in a dark RIKKEN work uniform and cap repairing a massive energy conduit deep under odaiba, blue-white core glow lighting her face from below, warm amber work lamps and CRT gauges around her, cathedral-scale machinery and thick cables, retro-futuristic evangelion atmosphere, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no fantasy armor, text, watermark</t>
+          <t>female engineer in dark work uniform riding an open elevator platform down a colossal glowing core shaft, hair blown upward, wrench on her shoulder, blue-white light rising from far below, amber safety beacons flashing past, league of legends splash art, highly detailed, dynamic composition, cinematic lighting --no fantasy armor, text, watermark</t>
         </is>
       </c>
     </row>
@@ -877,7 +877,7 @@
       </c>
       <c r="S4" s="5" t="inlineStr">
         <is>
-          <t>female operative in a sleek matte black high-tech exosuit with segmented mechanical armor plates like alita battle angel, thin water conduits glowing cyan along her forearms, fine mist condensing around her open hands, cyan key light from her own conduits on her face, warm sodium lights and thick cables in the concrete hall behind, retro-futuristic evangelion atmosphere, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no medieval knight armor, fantasy armor, ornate gold trim, text, watermark</t>
+          <t>female operative in a matte black segmented exosuit walking out of the sea at dawn, ribbons of water spiraling off her cyan-lit conduits, wet sand mirroring the pink sky, league of legends splash art, highly detailed, dynamic composition, cinematic lighting --no fantasy armor, medieval knight armor, text, watermark</t>
         </is>
       </c>
     </row>
@@ -960,7 +960,7 @@
       </c>
       <c r="S5" s="5" t="inlineStr">
         <is>
-          <t>female scout in a sleek matte black high-tech exosuit with segmented armor plates like alita battle angel, faint blue glowing seams, crouched on wooden scaffolding above a foggy 19th century parisian construction site at dusk, warm amber gaslight beside her illuminating her face, violet evening sky behind the iron beams, her futuristic suit the only modern element in the era, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no eiffel tower, medieval knight armor, fantasy armor, text, watermark</t>
+          <t>female scout in a matte black segmented exosuit leaping between wooden scaffolding beams above the rooftops of 1888 paris at sunrise, blue suit seams trailing, sea of fog below, golden light on iron beams, league of legends splash art, highly detailed, dynamic composition, cinematic lighting --no eiffel tower, fantasy armor, text, watermark</t>
         </is>
       </c>
     </row>
@@ -1043,7 +1043,7 @@
       </c>
       <c r="S6" s="5" t="inlineStr">
         <is>
-          <t>towering broad man in a heavy matte black segmented exosuit with thick mechanical shoulder plates, helmet off revealing a scarred stern face, arms crossed before a circular transfer platform, blue-white ring glow rising behind him, amber warning lights and thick cables on the brutalist concrete walls, retro-futuristic evangelion atmosphere, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no medieval knight armor, fantasy armor, giant robot, full helmet covering face, text, watermark</t>
+          <t>massive guard in a heavy matte black exosuit bracing wide-stance against a shockwave of blue light from an activating transfer platform, sparks streaming past him, his scarred face gritted and lit blue, amber alarms spinning, league of legends splash art, highly detailed, dynamic composition, cinematic lighting --no fantasy armor, giant robot, full helmet, text, watermark</t>
         </is>
       </c>
     </row>
@@ -1126,7 +1126,7 @@
       </c>
       <c r="S7" s="5" t="inlineStr">
         <is>
-          <t>stern analyst in a dark institutional uniform at a desk stacked with candidate files, round glasses reflecting pale blue light from a wall of CRT screens showing personnel records, warm amber desk lamp on his face, dark recruitment office at night with thick cables, retro-futuristic atmosphere, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no fantasy armor, cyberpunk pink purple, text, watermark</t>
+          <t>stern analyst with round glasses striding down a bright white archive hall, an armful of dossiers, loose pages flying behind him, holographic candidate faces flickering along the walls, cold daylight with one red rejected stamp, league of legends splash art, highly detailed, dynamic composition, cinematic lighting --no fantasy armor, text, watermark</t>
         </is>
       </c>
     </row>
@@ -1201,7 +1201,7 @@
       </c>
       <c r="S8" s="5" t="inlineStr">
         <is>
-          <t>human silhouette dissolving upward into a column of blue-white light on a circular transfer platform, a dropped coffee mug still falling where the person stood, dark empty facility hall with CRT control panels and amber standby lights, the light column blazing as the only bright source, retro-futuristic evangelion atmosphere, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, atmospheric detailed background --no fantasy magic portal, text, watermark</t>
+          <t>a runner dissolving into ascending blue-white light streaks mid-stride on a busy 2049 tokyo crosswalk in daylight, pedestrians turning in shock, his coffee cup suspended mid-air, league of legends splash art, highly detailed, dynamic composition, cinematic lighting --no fantasy magic, text, watermark</t>
         </is>
       </c>
     </row>
@@ -1276,7 +1276,7 @@
       </c>
       <c r="S9" s="5" t="inlineStr">
         <is>
-          <t>holographic briefing table projecting layered blue maps of seven historical eras, gloved hands of unseen officers pointing at one blank unmapped region, warm amber light from scattered papers and cold coffee cups, dark war-room with CRT screens and thick cables, retro-futuristic evangelion atmosphere, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, atmospheric detailed background --no fantasy magic, text, watermark</t>
+          <t>top-down view of officers standing on a glass floor above a huge rotating holographic map of seven historical eras, one era glowing blank and white, coffee cups and files scattered on the glass, blue glow lighting them from below, league of legends splash art, highly detailed, cinematic lighting --no fantasy magic, text, watermark</t>
         </is>
       </c>
     </row>
@@ -1361,7 +1361,7 @@
       </c>
       <c r="S10" s="5" t="inlineStr">
         <is>
-          <t>young franco-senegalese woman medic kneeling beside a wounded soldier in a dark field hospital tent, open palm emitting soft cyan light from fine diffuser pores in her matte black segmented exosuit glove, cyan conduits glowing along her forearm, warm lantern light against the cyan glow on her calm face, green CRT medical monitors behind her, retro-futuristic atmosphere, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no medieval knight armor, fantasy armor, text, watermark</t>
+          <t>young franco-senegalese medic in a matte black segmented exosuit running through warm rain carrying a wounded soldier on her back, her palm glowing cyan against his chest, field camp lanterns smearing in the wet dusk, league of legends splash art, highly detailed, dynamic composition, cinematic lighting --no fantasy armor, text, watermark</t>
         </is>
       </c>
     </row>
@@ -1446,7 +1446,7 @@
       </c>
       <c r="S11" s="5" t="inlineStr">
         <is>
-          <t>young japanese woman in a sleek matte black high-tech exosuit with segmented armor plates like alita battle angel, wide HUD visor over her eyes reflecting cascading blue probability data, standing in a dark analysis room lit by a wall of CRT screens, deep blue key light on her face, amber standby lights and thick cables in the background, retro-futuristic evangelion atmosphere, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no medieval knight armor, fantasy armor, ornate gold trim, text, watermark</t>
+          <t>young japanese woman in a matte black segmented exosuit standing on the top beam of a radio tower at dawn, wind whipping her hair, HUD visor streaming blue data against the pale gold sky, clouds far below, league of legends splash art, highly detailed, cinematic lighting --no fantasy armor, text, watermark</t>
         </is>
       </c>
     </row>
@@ -1513,7 +1513,7 @@
       </c>
       <c r="S12" s="5" t="inlineStr">
         <is>
-          <t>male traveler in a sleek matte black segmented exosuit like alita battle angel with contained ember-orange combustion channels along his arms and shoulders, heat shimmer rising from his gauntlets, embers drifting in a dark testing chamber, warm orange key light from his own conduits on his calm face, cool teal shadows and CRT monitors behind, retro-futuristic atmosphere, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no medieval knight armor, fantasy armor, fire everywhere, text, watermark</t>
+          <t>male traveler in a matte black segmented exosuit sprinting up a collapsing stairwell, ember-orange channels blazing along his arms, burning debris falling around him, cool blue smoke above, league of legends splash art, highly detailed, dynamic composition, cinematic lighting --no fantasy armor, fire everywhere, text, watermark</t>
         </is>
       </c>
     </row>
@@ -1596,7 +1596,7 @@
       </c>
       <c r="S13" s="5" t="inlineStr">
         <is>
-          <t>veteran traveler with grey temples in a heavy matte black segmented exosuit with thick worn armor plates and old mission scars, standing protectively in a steel doorway, warm amber corridor light behind him, faint blue glowing seams on his suit, tired unshakable eyes lit by a cool overhead lamp, brutalist concrete and thick cables, retro-futuristic atmosphere, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no medieval knight armor, fantasy armor, ornate gold trim, text, watermark</t>
+          <t>grey-templed veteran in a scarred matte black exosuit bracing his shoulder against a buckling steel door, impact flare blooming through the gap, debris flying past him, his blue seams flickering under the strain, league of legends splash art, highly detailed, dynamic composition, cinematic lighting --no fantasy armor, text, watermark</t>
         </is>
       </c>
     </row>
@@ -1671,7 +1671,7 @@
       </c>
       <c r="S14" s="5" t="inlineStr">
         <is>
-          <t>a man in 2049 civilian clothes being pulled off his feet toward a blazing column of blue-white light, one arm already dissolving into particles of light, terrified face turned toward the viewer, dark transfer chamber with CRT control panels flashing red alerts, thick cables whipping toward the column, retro-futuristic evangelion atmosphere, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no fantasy magic portal, text, watermark</t>
+          <t>a man in civilian clothes yanked off his feet toward a blazing blue-white light column, one arm dissolving into particles, terrified eyes meeting the viewer, morning light through tall lab windows, red alerts blinking, league of legends splash art, highly detailed, dynamic composition, cinematic lighting --no fantasy magic, text, watermark</t>
         </is>
       </c>
     </row>
@@ -1746,7 +1746,7 @@
       </c>
       <c r="S15" s="5" t="inlineStr">
         <is>
-          <t>translucent blue energy dome protecting a squad of travelers in matte black segmented exosuits kneeling on a transfer platform, warm amber sparks flaring where impacts hit the dome surface, dark brutalist hall with CRT panels and cables beyond, the dome glow lighting the squad from above, retro-futuristic evangelion atmosphere, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, atmospheric detailed background --no medieval knight armor, fantasy armor, creatures, monsters, text, watermark</t>
+          <t>squad of travelers in matte black exosuits kneeling under a translucent blue energy dome in a raging desert sandstorm, ancient arrows and debris shattering against the shield in amber bursts, league of legends splash art, highly detailed, dynamic composition, cinematic lighting --no fantasy armor, creatures, text, watermark</t>
         </is>
       </c>
     </row>
@@ -1813,7 +1813,7 @@
       </c>
       <c r="S16" s="5" t="inlineStr">
         <is>
-          <t>female squad coordinator in a dark RIKKEN officer uniform standing before a wall of CRT mission screens showing three teams in three different eras, headset on, one hand raised mid-order, pale blue monitor light on her face, warm amber comm lights and thick cables around the dark control room, retro-futuristic evangelion atmosphere, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no fantasy armor, text, watermark</t>
+          <t>female coordinator in dark officer uniform leaning over the rail of a floating gantry, pointing sharply, a ring of giant mission screens glowing around her showing three different eras, blue light from below and amber comm lights, league of legends splash art, highly detailed, cinematic lighting --no fantasy armor, text, watermark</t>
         </is>
       </c>
     </row>
@@ -1902,7 +1902,7 @@
       </c>
       <c r="S17" s="5" t="inlineStr">
         <is>
-          <t>young russian traveler with slicked blond hair grinning insolently, crouched low on a rooftop edge ready to launch, orange combustion glow flaring from the calf conduits of his matte black segmented exosuit like alita battle angel, orange key light from his own conduits on his face, teal-shadowed 2049 tokyo skyline with distant neon signs behind him, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no medieval knight armor, fantasy armor, fire everywhere, ornate gold trim, text, watermark</t>
+          <t>young russian traveler grinning mid-leap high between two rooftops, orange nitro flames roaring from his calf conduits, 2049 tokyo spread far below in teal evening haze, his silhouette against the blazing sunset, league of legends splash art, highly detailed, dynamic composition, cinematic lighting --no fantasy armor, text, watermark</t>
         </is>
       </c>
     </row>
@@ -1987,7 +1987,7 @@
       </c>
       <c r="S18" s="5" t="inlineStr">
         <is>
-          <t>traveler in a sleek matte black segmented exosuit like alita battle angel standing in a foggy historical battlefield, rusted iron debris and broken blades levitating in a slow orbit around him, pale blue glowing seams lighting his face from below, warm bronze fog and eroded earthworks behind, his futuristic suit the only modern element in the era, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no medieval knight armor, fantasy armor, fantasy magic, text, watermark</t>
+          <t>traveler in a matte black segmented exosuit walking slowly across a cratered ancient battlefield as thousands of rusted blades and iron shards rise from the mud around him like reversed rain, bronze fog, his blue seams the only cold light, league of legends splash art, highly detailed, cinematic lighting --no fantasy armor, fantasy magic, text, watermark</t>
         </is>
       </c>
     </row>
@@ -2062,7 +2062,7 @@
       </c>
       <c r="S19" s="5" t="inlineStr">
         <is>
-          <t>colossal underground transfer core beneath tokyo blazing with blue-white overload, tiny engineers running on steel gantries silhouetted against the light, cathedral-scale machinery with thick cables and amber warning strobes, steam venting from brutalist concrete walls, retro-futuristic evangelion industrial atmosphere, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, atmospheric detailed background --no fantasy magic, spaceship, explosion, text, watermark</t>
+          <t>vertical view up the throat of a colossal energy core mid-overload, rings of machinery blazing blue-white, engineers zip-lining away on cables, steam and amber strobes, industrial cathedral scale, league of legends splash art, highly detailed, dynamic composition, cinematic lighting --no spaceship, explosion, text, watermark</t>
         </is>
       </c>
     </row>
@@ -2129,7 +2129,7 @@
       </c>
       <c r="S20" s="5" t="inlineStr">
         <is>
-          <t>stern japanese woman in her fifties in an impeccable dark RIKKEN uniform seated at an elevated jury desk in a white immaculate test center, evaluating gaze cutting down at the viewer, cold clinical white key light on her face, one glowing blue insignia on her collar, warm amber file lamps on the desk, subject in the upper half of the frame, lower third calm and atmospheric, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no fantasy armor, text, watermark</t>
+          <t>stern japanese woman in an impeccable dark uniform standing in a vast white amphitheater as hundreds of holographic candidate portraits flicker out around her, only three still lit, her red pen paused over a list, cold daylight, league of legends splash art, highly detailed, cinematic lighting --no fantasy armor, text, watermark</t>
         </is>
       </c>
     </row>
@@ -2218,7 +2218,7 @@
       </c>
       <c r="S21" s="5" t="inlineStr">
         <is>
-          <t>imposing japanese man in his sixties with a granite face and grey brush cut wearing a first-generation exosuit with patinated copper conductors, thick old-school plates and mechanical piston joints, standing like a rock in a dark hangar, warm brass key light from his suit's aged conductors on his face, cool blue hangar lights and thick cables behind, subject in the upper half of the frame, lower third atmospheric, retro-futuristic atmosphere, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no medieval knight armor, fantasy armor, ornate gold trim, text, watermark</t>
+          <t>huge japanese man in his sixties charging through a collapsing wall in a first-generation exosuit of patinated copper and brass, steam pistons venting, rubble bouncing off his shoulders, warm brass light through the dust, league of legends splash art, highly detailed, dynamic composition, cinematic lighting --no medieval knight armor, fantasy armor, text, watermark</t>
         </is>
       </c>
     </row>
@@ -2285,7 +2285,7 @@
       </c>
       <c r="S22" s="5" t="inlineStr">
         <is>
-          <t>broad-shouldered chinese man in a heavy matte black segmented exosuit like alita battle angel, forearm and chest plates condensed into liquid-stone density, one massive fist wrapped in a subtle compressive distortion, cracked concrete radiating under his feet in a dark testing arena, blue key light from arena floodlights on his face, warm dust haze behind, subject in the upper half of the frame, lower third atmospheric, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no medieval knight armor, fantasy armor, hulk, giant robot, text, watermark</t>
+          <t>broad-shouldered chinese man in a heavy matte black exosuit frozen at the instant his fist meets a flooded arena floor, a crown of water erupting around the impact, shockwave rings in the shallow water, floodlights refracting through the spray, league of legends splash art, highly detailed, dynamic composition, cinematic lighting --no fantasy armor, hulk, text, watermark</t>
         </is>
       </c>
     </row>
@@ -2374,7 +2374,7 @@
       </c>
       <c r="S23" s="5" t="inlineStr">
         <is>
-          <t>19 year old slim french-japanese young man with light beige tousled hair, one single vivid red strand over his right brow and a thin scar on his right cheekbone, standing at the center of a transfer platform in a sleek matte black prototype exosuit with modular reconfiguring panels, a small engraved golden circle glowing on his chest, blue-white light column rising behind him, blue key light on his determined face, CRT monitors and thick cables around the platform ring, subject in the upper half of the frame, lower third atmospheric, retro-futuristic evangelion atmosphere, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no medieval knight armor, fantasy armor, ornate gold trim, text, watermark</t>
+          <t>19 year old french-japanese young man with light beige hair and one red strand falling backward through a shattering sky of seven eras, fragments showing paris scaffolds, snowy trenches, feudal bridges and ice seas, his prototype exosuit syncing with multi-hued light, calm eyes reaching upward, golden circle glowing on his chest, league of legends splash art, highly detailed, dynamic composition, cinematic lighting --no fantasy armor, text, watermark</t>
         </is>
       </c>
     </row>
@@ -2457,7 +2457,7 @@
       </c>
       <c r="S24" s="5" t="inlineStr">
         <is>
-          <t>unremarkable middle-aged agent in a dark RIKKEN staff uniform standing in a facility corridor at 3am, authentic institute badge on his chest, half his face in shadow, one tiny red LED reflected in his eye, cold blue corridor light and a distant red security light down the hall, CRT panels and thick cables on the walls, retro-futuristic blade runner atmosphere, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no fantasy armor, text, watermark</t>
+          <t>unremarkable agent in RIKKEN staff uniform walking through a crowded bright lobby, every other person motion-blurred, his badge catching a tiny red glint, cold daylight through glass, league of legends splash art, highly detailed, cinematic lighting --no fantasy armor, text, watermark</t>
         </is>
       </c>
     </row>
@@ -2524,7 +2524,7 @@
       </c>
       <c r="S25" s="5" t="inlineStr">
         <is>
-          <t>young candidate in recruit fatigues standing in line at the white RIKKEN test center, posture identical to the others but eyes measuring the room like a professional, thin red thread bracelet under his sleeve, cold clinical white key light, other candidates softly blurred around him, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no fantasy armor, text, watermark</t>
+          <t>young candidate sprinting a fitness test among other recruits in a bright training hall, all straining except him, effortless, eyes sliding sideways toward the viewer, one thin red thread bracelet, harsh white light, league of legends splash art, highly detailed, dynamic composition, cinematic lighting --no fantasy armor, text, watermark</t>
         </is>
       </c>
     </row>
@@ -2591,7 +2591,7 @@
       </c>
       <c r="S26" s="5" t="inlineStr">
         <is>
-          <t>operative in a stolen matte black segmented exosuit moving silently through an empty facility corridor at night, suit seams flickering red and miscalibrated, one hand trailing along the wall, a dead security camera behind him, cold blue emergency lighting with his red seams as the warm counterpoint, brutalist concrete and cables, retro-futuristic blade runner atmosphere, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no medieval knight armor, fantasy armor, text, watermark</t>
+          <t>operative in a stolen matte black exosuit dropping from a ceiling vent into a server aisle, coat flaring, red miscalibrated seams sputtering, cool blue server glow below him, league of legends splash art, highly detailed, dynamic composition, cinematic lighting --no fantasy armor, text, watermark</t>
         </is>
       </c>
     </row>
@@ -2658,7 +2658,7 @@
       </c>
       <c r="S27" s="5" t="inlineStr">
         <is>
-          <t>patient watcher in dark 2049 civilian clothes standing on a rooftop overlooking tokyo bay at night, binoculars lowered, wind in his coat, the city lights muted and grey except one distant red aircraft beacon, cool blue night key light on his face with the red beacon reflected in his eyes, retro-futuristic blade runner atmosphere, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no fantasy armor, cyberpunk pink purple overload, text, watermark</t>
+          <t>patient watcher in dark civilian clothes sitting on the roof of a ferris wheel cabin at dusk over tokyo bay, binoculars resting on his knee, wind in his coat, the fairground lights violet and gold below, one red beacon blinking far across the water, league of legends splash art, highly detailed, cinematic lighting --no fantasy armor, text, watermark</t>
         </is>
       </c>
     </row>
@@ -2741,7 +2741,7 @@
       </c>
       <c r="S28" s="5" t="inlineStr">
         <is>
-          <t>kairos fighter in a mismatched stolen exosuit with segmented panels from different CELL generations bolted together, red seams sputtering and glitching, aggressive hunched stance in a dark parking structure, red key light from his own faulty conduits on his face, warm sodium lights and thick pillars behind, retro-futuristic blade runner atmosphere, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no medieval knight armor, fantasy armor, text, watermark</t>
+          <t>kairos fighter in a mismatched bolted exosuit charging straight at the viewer down a parking ramp, sparks bursting from misfiring red calf conduits, sodium lights streaking overhead, league of legends splash art, highly detailed, dynamic composition, cinematic lighting --no fantasy armor, text, watermark</t>
         </is>
       </c>
     </row>
@@ -2808,7 +2808,7 @@
       </c>
       <c r="S29" s="5" t="inlineStr">
         <is>
-          <t>cold professional woman in a tailored dark coat standing over an open briefcase of precise tech instruments, surgical calm, dark hotel room with the muted tokyo night skyline behind glass, one red instrument light on her face against cool blue window light, retro-futuristic blade runner atmosphere, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no fantasy armor, blood, text, watermark</t>
+          <t>cold professional woman in a tailored coat walking away from a hotel entrance through light rain, steel case in hand, neon reds and cyans smearing in the wet street around her unhurried stride, league of legends splash art, highly detailed, cinematic lighting --no fantasy armor, blood, text, watermark</t>
         </is>
       </c>
     </row>
@@ -2875,7 +2875,7 @@
       </c>
       <c r="S30" s="5" t="inlineStr">
         <is>
-          <t>executive in an impeccable suit standing in a glass corner office above tokyo at night, back to the viewer, his unreadable face reflected in the window, red seal stamp resting on signed documents, warm desk lamp against the cool blue city glow, retro-futuristic blade runner atmosphere, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no fantasy armor, text, watermark</t>
+          <t>executive signing documents at a boardroom table in golden hour light high above tokyo, his fountain pen scratching, a faint red emergency glow from the city reflected in the glass behind him, league of legends splash art, highly detailed, cinematic lighting --no fantasy armor, text, watermark</t>
         </is>
       </c>
     </row>
@@ -2942,7 +2942,7 @@
       </c>
       <c r="S31" s="5" t="inlineStr">
         <is>
-          <t>close-up of a gloved hand sliding a thin red-sealed dossier across a polished dark table toward a trembling bare hand, tea untouched, faces out of frame, warm lamp light pooling on the table with the red seal as the sharpest color, dark meeting room with a CRT glowing in the background, retro-futuristic atmosphere, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the hands, atmospheric detailed background --no fantasy magic, text, watermark</t>
+          <t>close-up of a gloved hand passing a red-sealed dossier between seats of a moving maglev train, countryside smearing past the window in morning light, the other hand hesitating, league of legends splash art, highly detailed, cinematic lighting --no fantasy magic, text, watermark</t>
         </is>
       </c>
     </row>
@@ -3009,7 +3009,7 @@
       </c>
       <c r="S32" s="5" t="inlineStr">
         <is>
-          <t>circular transfer platform short-circuiting in a dark hall, its blue ring guttering out while red warning strobes sweep the walls, sparks raining from severed thick cables, a small sabotage device blinking red at the platform base, no people, CRT panels flashing errors, retro-futuristic evangelion atmosphere, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, atmospheric detailed background --no fantasy magic, explosion, text, watermark</t>
+          <t>silhouette walking calmly toward the viewer as a transfer platform erupts in blue sparks and dying light behind, red strobes sweeping the smoke, shards raining, league of legends splash art, highly detailed, dynamic composition, cinematic lighting --no explosion fireball, text, watermark</t>
         </is>
       </c>
     </row>
@@ -3076,7 +3076,7 @@
       </c>
       <c r="S33" s="5" t="inlineStr">
         <is>
-          <t>female kairos operative in a dark tech coat over a matte black segmented exosuit raising a small parasite emitter, translucent red interference waves rippling from it, a distant traveler's blue suit seams visibly stuttering and dying, red key light from the emitter on her focused face, dark facility hall with cables and CRT panels, retro-futuristic blade runner atmosphere, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no medieval knight armor, fantasy armor, text, watermark</t>
+          <t>female kairos operative crouched on the roof of a speeding maglev at night deploying a red pulse emitter, the interference wave rippling backward along the train as blue window lights die car by car, wind tearing at her coat, league of legends splash art, highly detailed, dynamic composition, cinematic lighting --no fantasy armor, text, watermark</t>
         </is>
       </c>
     </row>
@@ -3143,7 +3143,7 @@
       </c>
       <c r="S34" s="5" t="inlineStr">
         <is>
-          <t>lean duelist in a stolen matte black segmented exosuit like alita battle angel, contained electric arcs crawling between his gauntlets, red-tinged capacitor seams pulsing along his spine, combat stance in a rain-slick dark alley, white-blue arc light on his face against the red seams, cyan reflections in the puddles, retro-futuristic blade runner atmosphere, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no medieval knight armor, fantasy armor, lightning storm, text, watermark</t>
+          <t>lean duelist in a stolen matte black exosuit lunging across a rain-flooded intersection at night, white-blue arc light trailing his gauntlet, red capacitor seams blazing down his spine, neon reflections shattering under his splash, league of legends splash art, highly detailed, dynamic composition, cinematic lighting --no fantasy armor, lightning storm, text, watermark</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3210,7 @@
       </c>
       <c r="S35" s="5" t="inlineStr">
         <is>
-          <t>charming recruiter in RIKKEN colors leaning across an interview table toward an unseen candidate, warm practiced smile that stops below the eyes, red pen turning slowly between his fingers, warm desk lamp on his face against the cool dark interview room, a CRT recorder blinking in the corner, retro-futuristic atmosphere, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no fantasy armor, text, watermark</t>
+          <t>charming recruiter guiding a nervous candidate down a bright corridor, arm around his shoulder, practiced warm smile, a red pen spinning in his free hand behind his back, morning light, league of legends splash art, highly detailed, cinematic lighting --no fantasy armor, text, watermark</t>
         </is>
       </c>
     </row>
@@ -3277,7 +3277,7 @@
       </c>
       <c r="S36" s="5" t="inlineStr">
         <is>
-          <t>huge enforcer in a reinforced matte black segmented exosuit filling a narrow basement corridor, head bowed under the ceiling, knuckles wrapped in red-lit compression bands, steam from pipes catching the red glow, warm sodium light behind him and cold shadows ahead, brutalist concrete and thick cables, retro-futuristic atmosphere, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no medieval knight armor, fantasy armor, hulk, giant robot, text, watermark</t>
+          <t>huge enforcer in a reinforced matte black exosuit shouldering through a concrete wall, rebar bending around him, dust exploding into shafts of basement sunlight, red compression bands glowing on his knuckles, league of legends splash art, highly detailed, dynamic composition, cinematic lighting --no fantasy armor, hulk, giant robot, text, watermark</t>
         </is>
       </c>
     </row>
@@ -3344,7 +3344,7 @@
       </c>
       <c r="S37" s="5" t="inlineStr">
         <is>
-          <t>a traveler's matte black exosuit mid-activation abruptly failing, its blue glowing seams shattering into static as a translucent red interference wave passes through the frame, the traveler's silhouette frozen mid-gesture in a dark hall, blue light dying into red across the scene, CRT panels glitching behind, retro-futuristic evangelion atmosphere, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, atmospheric detailed background --no fantasy magic, text, watermark</t>
+          <t>a traveler stumbling mid-sprint as his blue suit seams shatter into static, a translucent red wave passing through the frame, his momentum carrying him toward the ground, dusk street, league of legends splash art, highly detailed, dynamic composition, cinematic lighting --no fantasy magic, text, watermark</t>
         </is>
       </c>
     </row>
@@ -3411,7 +3411,7 @@
       </c>
       <c r="S38" s="5" t="inlineStr">
         <is>
-          <t>human figure being torn backward out of a warm historical street scene into red-black static, fingers clawing at air, the era continuing undisturbed around the void he leaves, warm bronze daylight in the scene against the cold red-black tear, sense of violent temporal removal, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no fantasy magic portal, gore, text, watermark</t>
+          <t>man yanked backward off his feet into a tear of red-black static above a sunlit historical market street, fruit scattering from a knocked stall, bystanders frozen unaware, warm bronze daylight against the cold red tear, league of legends splash art, highly detailed, dynamic composition, cinematic lighting --no gore, text, watermark</t>
         </is>
       </c>
     </row>
@@ -3478,7 +3478,7 @@
       </c>
       <c r="S39" s="5" t="inlineStr">
         <is>
-          <t>female kairos agent in a stolen matte black segmented exosuit kneeling in a foggy blind-zone battlefield, prying a relic from the mud into a red-lit containment case, red case light on her hurried face against the warm bronze fog of the era, disturbed ancient earth around her, her modern suit profane against the historical dead ground, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no medieval knight armor, fantasy armor, gore, skeletons, text, watermark</t>
+          <t>female kairos agent sprinting out of a bronze fog battlefield clutching a red-lit relic case, mud kicking from her boots, ghostly still silhouettes of the era watching motionless from the mist behind her, league of legends splash art, highly detailed, dynamic composition, cinematic lighting --no fantasy armor, gore, text, watermark</t>
         </is>
       </c>
     </row>
@@ -3545,7 +3545,7 @@
       </c>
       <c r="S40" s="5" t="inlineStr">
         <is>
-          <t>interrogator in an immaculate dark uniform standing beside an empty steel chair in a blinding white interrogation room, his long shadow falling across the chair, one red recording light on the wall reflected in his glasses, cold white key light with the red light as the only color, quiet menace, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no fantasy armor, text, watermark</t>
+          <t>interrogator in an immaculate dark uniform circling an empty steel chair in a blinding white room, one gloved hand trailing along its back, his long shadow sweeping the floor, a single red recording light, league of legends splash art, highly detailed, cinematic lighting --no fantasy armor, text, watermark</t>
         </is>
       </c>
     </row>
@@ -3612,7 +3612,7 @@
       </c>
       <c r="S41" s="5" t="inlineStr">
         <is>
-          <t>kairos operative in a sleek stolen matte black segmented exosuit standing calmly while a swarm of palm-sized drones orbits him in a slow constellation, each drone eye a tiny red point, red drone lights rimming his silhouette against the cool blue glow of a dark server hall, thick cables and blinking racks behind, retro-futuristic blade runner atmosphere, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no medieval knight armor, fantasy armor, text, watermark</t>
+          <t>kairos operative standing on a data-center rooftop at night, arms open as his drone swarm spirals upward into a towering red constellation column above the city, cyan server glow venting from the roof hatches, league of legends splash art, highly detailed, dynamic composition, cinematic lighting --no fantasy armor, text, watermark</t>
         </is>
       </c>
     </row>
@@ -3679,7 +3679,7 @@
       </c>
       <c r="S42" s="5" t="inlineStr">
         <is>
-          <t>monumental cracked clock face suspended in darkness, thin red light bleeding through the fracture lines, a single silhouette stepping through the largest crack as through a door, cold grey clockwork detail against the red glow, subject in the upper half of the frame, lower third dark and atmospheric, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, atmospheric detailed background --no fantasy magic portal, text, watermark</t>
+          <t>silhouette leaping through a monumental shattering clock face, shards of glass and time exploding outward frozen mid-burst, thin red light bleeding through every crack, darkness beyond, league of legends splash art, highly detailed, dynamic composition, cinematic lighting --no fantasy magic portal, text, watermark</t>
         </is>
       </c>
     </row>
@@ -3762,7 +3762,7 @@
       </c>
       <c r="S43" s="5" t="inlineStr">
         <is>
-          <t>distinguished japanese director in his fifties in a flawless dark suit seated at a directorial desk high above the tokyo night, hands calmly folded, warm gentle smile slightly too perfect to be true, warm desk lamp key light on his face, red seal ring catching the light, cool blue city glow through the glass behind him, subject in the upper half of the frame, lower third atmospheric, retro-futuristic blade runner atmosphere, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no fantasy armor, villain sneer, text, watermark</t>
+          <t>distinguished japanese director descending a grand marble staircase amid an audience of standing shadowed figures applauding, only his warm too-perfect smile fully lit, red seal ring catching the chandelier light, league of legends splash art, highly detailed, cinematic lighting --no fantasy armor, villain sneer, text, watermark</t>
         </is>
       </c>
     </row>
@@ -3829,7 +3829,7 @@
       </c>
       <c r="S44" s="5" t="inlineStr">
         <is>
-          <t>austere woman in a dark tailored suit standing in a shadowed archive of ledgers and red-stamped files, holding a single page up into a thin blade of warm light, faces of debtors pinned on threads behind her like a silent web, warm amber blade of light on her face against the cold dark stacks, red stamps as the sharpest color, subject in the upper half of the frame, lower third atmospheric, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no fantasy armor, text, watermark</t>
+          <t>austere woman standing calm at the center of a slow cyclone of ledger pages in a shadowed vault, red-stamped sheets orbiting her, one page pinched precisely between two fingers, a blade of warm light cutting the dust, league of legends splash art, highly detailed, dynamic composition, cinematic lighting --no fantasy magic, text, watermark</t>
         </is>
       </c>
     </row>
@@ -3918,7 +3918,7 @@
       </c>
       <c r="S45" s="5" t="inlineStr">
         <is>
-          <t>tall gaunt japanese man with hollow calm eyes in a long black coat over a matte black segmented exosuit, standing in falling snow at night, one raised hand crushing a glowing blue CELL core that dies between his fingers, red glowing seams under the coat, sodium street lights and a flickering CRT billboard behind, brutalist government building in the snow haze, subject in the upper half of the frame, lower third atmospheric, retro-futuristic blade runner atmosphere, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no medieval knight armor, fantasy armor, cape flowing dramatically, text, watermark</t>
+          <t>gaunt japanese man in a long black coat over a matte black exosuit lunging through a night blizzard, twin adaptive blades extended, red seams blazing through the snow, a dying blue CELL core crushed in his trailing hand, sodium lights haloing the storm, league of legends splash art, highly detailed, dynamic composition, cinematic lighting --no fantasy armor, cape, text, watermark</t>
         </is>
       </c>
     </row>
@@ -3985,7 +3985,7 @@
       </c>
       <c r="S46" s="5" t="inlineStr">
         <is>
-          <t>street kid in patched wool clothes and an oversized cap standing in a fog-drowned parisian alley in 1888, sharp knowing eyes, warm gaslight from a lantern above him against the cool teal fog, iron scaffolding as vague shapes in the mist erasing every landmark, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no eiffel tower, modern elements, text, watermark</t>
+          <t>street kid in patched wool clothes sprinting across the rooftops of 1888 paris with a stolen loaf, pigeons bursting around him, chimney smoke and morning fog below, warm gaslight amber against cool blue slate roofs, league of legends splash art, highly detailed, dynamic composition, cinematic lighting --no eiffel tower, modern elements, text, watermark</t>
         </is>
       </c>
     </row>
@@ -4052,7 +4052,7 @@
       </c>
       <c r="S47" s="5" t="inlineStr">
         <is>
-          <t>laundress in rough 19th century workclothes wringing linen at a river bank at dawn, strong tired hands, her breath visible, warm bronze dawn light on her face through the thick fog that hides the far shore and every monument, cold blue-grey water, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no recognizable landmarks, modern elements, text, watermark</t>
+          <t>laundress in rough 19th century workclothes wading thigh-deep in a river at sunrise, hauling heavy linen against the current, spray catching the gold light, fog erasing the far shore, league of legends splash art, highly detailed, dynamic composition, cinematic lighting --no recognizable landmarks, modern elements, text, watermark</t>
         </is>
       </c>
     </row>
@@ -4127,7 +4127,7 @@
       </c>
       <c r="S48" s="5" t="inlineStr">
         <is>
-          <t>masterless samurai in worn dark travel clothes standing at the foot of a wooden bridge swallowed by river mist, hand resting on a chipped saya, warm lantern light from a post beside him against the cold teal mist, the far end of the bridge invisible, no banners no crest, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no famous castle, modern elements, text, watermark</t>
+          <t>masterless samurai mid-draw on a mist-drowned wooden bridge, blade a silver arc, river spray and maple leaves swirling, warm lantern light against the cold teal fog, league of legends splash art, highly detailed, dynamic composition, cinematic lighting --no famous castle, modern elements, text, watermark</t>
         </is>
       </c>
     </row>
@@ -4194,7 +4194,7 @@
       </c>
       <c r="S49" s="5" t="inlineStr">
         <is>
-          <t>weathered stonemason in medieval work clothes laying stones of a small unfinished mountain chapel as snow buries the pass, mallet in cracked hands, warm firelight from a brazier beside him against the blue whiteout erasing the valley below, creaking wooden scaffold, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no recognizable cathedral, modern elements, text, watermark</t>
+          <t>weathered stonemason hauling a stone block up a creaking rope pulley in driving snow, scaffold swaying against the unfinished mountain chapel, his brazier sparking orange in the blue whiteout, league of legends splash art, highly detailed, dynamic composition, cinematic lighting --no modern elements, text, watermark</t>
         </is>
       </c>
     </row>
@@ -4261,7 +4261,7 @@
       </c>
       <c r="S50" s="5" t="inlineStr">
         <is>
-          <t>lone roman legionary in mud-caked worn armor standing in a dark primeval forest, shield split, exhausted defiance on his rain-streaked face, pale bronze light breaking through colossal trees while fog swallows the rest of his column, moss green shadows, no standard visible, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no roman monument, modern elements, fantasy armor, text, watermark</t>
+          <t>lone roman legionary charging through giant ferns in a dark primeval forest, split shield raised, mud flying from his boots, pale bronze light breaking through the canopy onto his roaring face, fog swallowing everything behind, league of legends splash art, highly detailed, dynamic composition, cinematic lighting --no roman monument, modern elements, text, watermark</t>
         </is>
       </c>
     </row>
@@ -4328,7 +4328,7 @@
       </c>
       <c r="S51" s="5" t="inlineStr">
         <is>
-          <t>harpooner in heavy oilskins standing at the icy bow of a whaling boat locked in pack ice, harpoon planted, frost in his beard, warm oil lamp light on his face against the vast teal ice and the grey fog wall where sea and sky fuse, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no modern ships, text, watermark</t>
+          <t>harpooner in heavy oilskins hurling his harpoon from the icy bow as a wave bursts against the hull, spray freezing mid-air, teal icebergs and grey fog wall behind, his oil lantern swinging gold, league of legends splash art, highly detailed, dynamic composition, cinematic lighting --no modern ships, text, watermark</t>
         </is>
       </c>
     </row>
@@ -4395,7 +4395,7 @@
       </c>
       <c r="S52" s="5" t="inlineStr">
         <is>
-          <t>colossal prehistoric steppe bear rearing in a blizzard on an endless white plain, fur crusted with ice, breath like smoke, pale gold dawn light catching its silhouette against the blue snowstorm that erases the horizon, primal and indifferent, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no modern elements, text, watermark</t>
+          <t>colossal prehistoric steppe bear charging toward the viewer through a blizzard, snow exploding from each stride, ice-crusted fur, pale gold dawn cutting through the blue storm, league of legends splash art, highly detailed, dynamic composition, cinematic lighting --no modern elements, text, watermark</t>
         </is>
       </c>
     </row>
@@ -4462,7 +4462,7 @@
       </c>
       <c r="S53" s="5" t="inlineStr">
         <is>
-          <t>a bare human hand dissolving into drifting golden dust motes inside a single blade of late afternoon light, dark empty barn interior, the dust rising and scattering like memory, warm gold light against deep brown shadows, quiet and sad, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, atmospheric detailed background --no skeleton, gore, text, watermark</t>
+          <t>a bare hand dissolving into golden dust motes inside one blade of afternoon light, dark barn interior, the dust drifting upward like memory, league of legends splash art, highly detailed, cinematic lighting --no skeleton, gore, text, watermark</t>
         </is>
       </c>
     </row>
@@ -4529,7 +4529,7 @@
       </c>
       <c r="S54" s="5" t="inlineStr">
         <is>
-          <t>crowded historical tavern scene with every figure softly blurred except one perfectly sharp empty chair at the center table, a still-steaming cup before it, warm hearth light pooling on the empty seat against the cool blurred crowd, the absence louder than the noise, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, atmospheric detailed background --no modern elements, text, watermark</t>
+          <t>crowded historical tavern in warm hearth light, every figure softly blurred in motion except one perfectly sharp empty chair, a still-steaming cup before it, league of legends splash art, highly detailed, cinematic lighting --no modern elements, text, watermark</t>
         </is>
       </c>
     </row>
@@ -4596,7 +4596,7 @@
       </c>
       <c r="S55" s="5" t="inlineStr">
         <is>
-          <t>barefoot young messenger girl sprinting through a narrow ancient market street before dawn, sealed letter clutched to her chest, dust rising behind her heels, warm lantern glows in the awnings against the violet pre-dawn sky, no era landmark visible, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no modern elements, text, watermark</t>
+          <t>barefoot messenger girl sprinting low through a narrow ancient market street before dawn, sealed letter clutched to her chest, dust and startled doves in her wake, violet sky over warm lantern awnings, league of legends splash art, highly detailed, dynamic composition, cinematic lighting --no modern elements, text, watermark</t>
         </is>
       </c>
     </row>
@@ -4663,7 +4663,7 @@
       </c>
       <c r="S56" s="5" t="inlineStr">
         <is>
-          <t>old griot storyteller mid-tale at a night fire, hands spread wide casting long shadows, sparks rising like his words, warm fire light on his animated face against the deep blue night, circle of captivated listeners leaning in from the darkness, no monument no writing anywhere, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no modern elements, text, watermark</t>
+          <t>old griot mid-tale at a night fire, arms sweeping wide as the rising sparks swirl into fleeting shapes of warriors and rivers above the flames, entranced listeners leaning in from the deep blue dark, league of legends splash art, highly detailed, dynamic composition, cinematic lighting --no modern elements, text, watermark</t>
         </is>
       </c>
     </row>
@@ -4730,7 +4730,7 @@
       </c>
       <c r="S57" s="5" t="inlineStr">
         <is>
-          <t>mountain woman warrior in furs and iron standing alone in a snowstorm at a narrow alpine pass, long spear planted, ice in her braids, immovable calm, warm bronze light from a watch fire beside her against the blue whiteout that erases the path behind, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no fantasy armor, ornate gold trim, modern elements, text, watermark</t>
+          <t>mountain woman warrior sweeping her long spear in a wide arc through the snowstorm at a narrow alpine pass, snow carving off the blade's path, furs whipping, warm watch-fire light against the blue whiteout, league of legends splash art, highly detailed, dynamic composition, cinematic lighting --no fantasy armor, modern elements, text, watermark</t>
         </is>
       </c>
     </row>
@@ -4797,7 +4797,7 @@
       </c>
       <c r="S58" s="5" t="inlineStr">
         <is>
-          <t>wide historical landscape whose center is simply unwritten, a soft pale void swallowing the middle of the scene, the world fraying into nothing at its edges, birds flying around the absence, warm bronze countryside against the cold blank void, eerie and calm, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, atmospheric detailed background --no fantasy magic portal, modern elements, text, watermark</t>
+          <t>wide historical landscape whose center is simply unwritten, a soft pale void swallowing the middle of the scene, birds wheeling around the absence, warm bronze countryside fraying into blank nothing, league of legends splash art, highly detailed, cinematic lighting --no fantasy magic portal, modern elements, text, watermark</t>
         </is>
       </c>
     </row>
@@ -4864,7 +4864,7 @@
       </c>
       <c r="S59" s="5" t="inlineStr">
         <is>
-          <t>lean swordsman in dark simple garb waiting at the far end of a mist-drowned wooden bridge, blade still sheathed, one hand raised in silent invitation, coiled stillness, cold steel-blue mist with a warm paper lantern glow at his feet, the river fog erasing everything beyond ten paces, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no famous landmark, modern elements, text, watermark</t>
+          <t>lean swordsman sprinting across the planks of a mist-drowned bridge toward the viewer, scabbard flung aside spinning mid-air, blade low and trailing, cold steel mist parting around him, one warm lantern flare, league of legends splash art, highly detailed, dynamic composition, cinematic lighting --no famous landmark, modern elements, text, watermark</t>
         </is>
       </c>
     </row>
@@ -4931,7 +4931,7 @@
       </c>
       <c r="S60" s="5" t="inlineStr">
         <is>
-          <t>early 1900s battleship emerging half-real from a wall of sea fog, hull streaked with rust, gun turrets silent, no flag identifiable, warm rust and bronze tones of the hull against the cold teal fog actively swallowing its stern as if unwriting it, heavy dark sea, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, atmospheric detailed background --no modern warships, explosion, text, watermark</t>
+          <t>early 1900s battleship bursting its rusted prow through a wall of sea fog toward the viewer, bow wave exploding, no flag, the fog visibly unwriting its stern into nothing, cold teal sea and warm rust, league of legends splash art, highly detailed, dynamic composition, cinematic lighting --no modern warships, text, watermark</t>
         </is>
       </c>
     </row>
@@ -4998,7 +4998,7 @@
       </c>
       <c r="S61" s="5" t="inlineStr">
         <is>
-          <t>ageless figure in layered robes from no single era standing in an impossible library where shelves curve into fog, holding an open book whose pages are blank, face half-lost in shadow beneath a deep hood, warm golden dust motes orbiting like slow time against the cold violet fog between the shelves, subject in the upper half of the frame, lower third atmospheric, league of legends splash art style, highly detailed semi-realistic digital illustration, dramatic cinematic lighting, sharp focus on the subject, atmospheric detailed background --no wizard fantasy, glowing runes, modern elements, text, watermark</t>
+          <t>ageless hooded figure looking up from an open blank book as thousands of books spiral upward around him into a vortex of golden dust and violet fog, impossible curved shelves dissolving into the sky, league of legends splash art, highly detailed, dynamic composition, cinematic lighting --no wizard fantasy, glowing runes, modern elements, text, watermark</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: Porteur CELL Pyros (R11) — 4⚡ 4/4 Synchro(2) Surchauffe 3 dégâts, art principal + 2 alternatifs
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/SET01-production.xlsx
+++ b/docs/SET01-production.xlsx
@@ -1461,9 +1461,9 @@
           <t>porteur-cell-pyros</t>
         </is>
       </c>
-      <c r="C12" s="6" t="inlineStr">
-        <is>
-          <t>À générer</t>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Forgée</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
@@ -1484,13 +1484,31 @@
       <c r="G12" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="H12" s="2" t="inlineStr"/>
-      <c r="I12" s="2" t="inlineStr"/>
-      <c r="J12" s="2" t="inlineStr"/>
+      <c r="H12" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="I12" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>CELL Pyros</t>
+        </is>
+      </c>
       <c r="K12" s="5" t="inlineStr"/>
-      <c r="L12" s="2" t="inlineStr"/>
-      <c r="M12" s="5" t="inlineStr"/>
-      <c r="N12" s="5" t="inlineStr"/>
+      <c r="L12" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="M12" s="5" t="inlineStr">
+        <is>
+          <t>Surchauffe : infligez 3 dégâts à une unité.</t>
+        </is>
+      </c>
+      <c r="N12" s="5" t="inlineStr">
+        <is>
+          <t>Le feu ne le brûle plus. C'est tout le reste qui brûle.</t>
+        </is>
+      </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
           <t>Non</t>

</xml_diff>

<commit_message>
feat: Coordinatrice d'escouade (R15) — 4⚡ 3/4 épique, vos Synchros coûtent (1) de moins
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/SET01-production.xlsx
+++ b/docs/SET01-production.xlsx
@@ -1779,9 +1779,9 @@
           <t>coordinatrice-descouade</t>
         </is>
       </c>
-      <c r="C16" s="6" t="inlineStr">
-        <is>
-          <t>À générer</t>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>Forgée</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
@@ -1802,13 +1802,29 @@
       <c r="G16" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="H16" s="2" t="inlineStr"/>
-      <c r="I16" s="2" t="inlineStr"/>
-      <c r="J16" s="2" t="inlineStr"/>
-      <c r="K16" s="5" t="inlineStr"/>
+      <c r="H16" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I16" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>CELL de série · Relais</t>
+        </is>
+      </c>
+      <c r="K16" s="5" t="inlineStr">
+        <is>
+          <t>Vos Synchros coûtent (1) de moins.</t>
+        </is>
+      </c>
       <c r="L16" s="2" t="inlineStr"/>
       <c r="M16" s="5" t="inlineStr"/>
-      <c r="N16" s="5" t="inlineStr"/>
+      <c r="N16" s="5" t="inlineStr">
+        <is>
+          <t>Trois équipes, trois siècles, une seule voix dans l'oreillette.</t>
+        </is>
+      </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
           <t>Non</t>

</xml_diff>

<commit_message>
feat: Yuriko Watanabe (R19) — légendaire 5⚡ 3/5, pioche de fin de tour, CELL 1re génération éteint (pas de Synchro)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/SET01-production.xlsx
+++ b/docs/SET01-production.xlsx
@@ -2111,9 +2111,9 @@
           <t>yuriko-watanabe</t>
         </is>
       </c>
-      <c r="C20" s="6" t="inlineStr">
-        <is>
-          <t>À générer</t>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>Forgée</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
@@ -2134,16 +2134,32 @@
       <c r="G20" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="H20" s="2" t="inlineStr"/>
-      <c r="I20" s="2" t="inlineStr"/>
-      <c r="J20" s="2" t="inlineStr"/>
-      <c r="K20" s="5" t="inlineStr"/>
+      <c r="H20" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I20" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>CELL 1re génération · éteint</t>
+        </is>
+      </c>
+      <c r="K20" s="5" t="inlineStr">
+        <is>
+          <t>À la fin de votre tour, piochez une carte.</t>
+        </is>
+      </c>
       <c r="L20" s="2" t="inlineStr"/>
       <c r="M20" s="5" t="inlineStr"/>
-      <c r="N20" s="5" t="inlineStr"/>
+      <c r="N20" s="5" t="inlineStr">
+        <is>
+          <t>Elle connaît le prix de chaque nom sur le mur. Elle signe quand même.</t>
+        </is>
+      </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
-          <t>Oui</t>
+          <t>Non</t>
         </is>
       </c>
       <c r="P20" s="2" t="inlineStr">

</xml_diff>

<commit_message>
feat: Liang Chen (R21) — légendaire 7⚡ 6/7 CELL Brutus, Synchro(3) Onde de choc 2 dégâts AoE, + 1 art alternatif
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/SET01-production.xlsx
+++ b/docs/SET01-production.xlsx
@@ -135,10 +135,10 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -2142,7 +2142,7 @@
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>CELL 1re génération · éteint</t>
+          <t>CELL 1G · éteint</t>
         </is>
       </c>
       <c r="K20" s="5" t="inlineStr">
@@ -2283,9 +2283,9 @@
           <t>liang-chen</t>
         </is>
       </c>
-      <c r="C22" s="6" t="inlineStr">
-        <is>
-          <t>À générer</t>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>Forgée</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
@@ -2306,16 +2306,34 @@
       <c r="G22" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="H22" s="2" t="inlineStr"/>
-      <c r="I22" s="2" t="inlineStr"/>
-      <c r="J22" s="2" t="inlineStr"/>
+      <c r="H22" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="I22" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>CELL Brutus</t>
+        </is>
+      </c>
       <c r="K22" s="5" t="inlineStr"/>
-      <c r="L22" s="2" t="inlineStr"/>
-      <c r="M22" s="5" t="inlineStr"/>
-      <c r="N22" s="5" t="inlineStr"/>
+      <c r="L22" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="M22" s="5" t="inlineStr">
+        <is>
+          <t>Onde de choc : infligez 2 dégâts à toutes les unités adverses.</t>
+        </is>
+      </c>
+      <c r="N22" s="5" t="inlineStr">
+        <is>
+          <t>Le sol se souvient de chacun de ses pas.</t>
+        </is>
+      </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
-          <t>Oui</t>
+          <t>Non</t>
         </is>
       </c>
       <c r="P22" s="2" t="inlineStr">
@@ -2444,7 +2462,7 @@
           <t>Forgée</t>
         </is>
       </c>
-      <c r="D24" s="7" t="inlineStr">
+      <c r="D24" s="6" t="inlineStr">
         <is>
           <t>KAIROS</t>
         </is>
@@ -2522,12 +2540,12 @@
           <t>taupe-du-recrutement</t>
         </is>
       </c>
-      <c r="C25" s="6" t="inlineStr">
+      <c r="C25" s="7" t="inlineStr">
         <is>
           <t>À générer</t>
         </is>
       </c>
-      <c r="D25" s="7" t="inlineStr">
+      <c r="D25" s="6" t="inlineStr">
         <is>
           <t>KAIROS</t>
         </is>
@@ -2589,12 +2607,12 @@
           <t>executant-de-nuit</t>
         </is>
       </c>
-      <c r="C26" s="6" t="inlineStr">
+      <c r="C26" s="7" t="inlineStr">
         <is>
           <t>À générer</t>
         </is>
       </c>
-      <c r="D26" s="7" t="inlineStr">
+      <c r="D26" s="6" t="inlineStr">
         <is>
           <t>KAIROS</t>
         </is>
@@ -2656,12 +2674,12 @@
           <t>guetteur-du-moment</t>
         </is>
       </c>
-      <c r="C27" s="6" t="inlineStr">
+      <c r="C27" s="7" t="inlineStr">
         <is>
           <t>À générer</t>
         </is>
       </c>
-      <c r="D27" s="7" t="inlineStr">
+      <c r="D27" s="6" t="inlineStr">
         <is>
           <t>KAIROS</t>
         </is>
@@ -2728,7 +2746,7 @@
           <t>Forgée</t>
         </is>
       </c>
-      <c r="D28" s="7" t="inlineStr">
+      <c r="D28" s="6" t="inlineStr">
         <is>
           <t>KAIROS</t>
         </is>
@@ -2806,12 +2824,12 @@
           <t>nettoyeuse</t>
         </is>
       </c>
-      <c r="C29" s="6" t="inlineStr">
+      <c r="C29" s="7" t="inlineStr">
         <is>
           <t>À générer</t>
         </is>
       </c>
-      <c r="D29" s="7" t="inlineStr">
+      <c r="D29" s="6" t="inlineStr">
         <is>
           <t>KAIROS</t>
         </is>
@@ -2873,12 +2891,12 @@
           <t>cadre-corrompu</t>
         </is>
       </c>
-      <c r="C30" s="6" t="inlineStr">
+      <c r="C30" s="7" t="inlineStr">
         <is>
           <t>À générer</t>
         </is>
       </c>
-      <c r="D30" s="7" t="inlineStr">
+      <c r="D30" s="6" t="inlineStr">
         <is>
           <t>KAIROS</t>
         </is>
@@ -2940,12 +2958,12 @@
           <t>chantage</t>
         </is>
       </c>
-      <c r="C31" s="6" t="inlineStr">
+      <c r="C31" s="7" t="inlineStr">
         <is>
           <t>À générer</t>
         </is>
       </c>
-      <c r="D31" s="7" t="inlineStr">
+      <c r="D31" s="6" t="inlineStr">
         <is>
           <t>KAIROS</t>
         </is>
@@ -3007,12 +3025,12 @@
           <t>sabotage-de-plateforme</t>
         </is>
       </c>
-      <c r="C32" s="6" t="inlineStr">
+      <c r="C32" s="7" t="inlineStr">
         <is>
           <t>À générer</t>
         </is>
       </c>
-      <c r="D32" s="7" t="inlineStr">
+      <c r="D32" s="6" t="inlineStr">
         <is>
           <t>KAIROS</t>
         </is>
@@ -3074,12 +3092,12 @@
           <t>brouilleuse</t>
         </is>
       </c>
-      <c r="C33" s="6" t="inlineStr">
+      <c r="C33" s="7" t="inlineStr">
         <is>
           <t>À générer</t>
         </is>
       </c>
-      <c r="D33" s="7" t="inlineStr">
+      <c r="D33" s="6" t="inlineStr">
         <is>
           <t>KAIROS</t>
         </is>
@@ -3141,12 +3159,12 @@
           <t>duelliste-cell-tempest</t>
         </is>
       </c>
-      <c r="C34" s="6" t="inlineStr">
+      <c r="C34" s="7" t="inlineStr">
         <is>
           <t>À générer</t>
         </is>
       </c>
-      <c r="D34" s="7" t="inlineStr">
+      <c r="D34" s="6" t="inlineStr">
         <is>
           <t>KAIROS</t>
         </is>
@@ -3208,12 +3226,12 @@
           <t>recruteur-double</t>
         </is>
       </c>
-      <c r="C35" s="6" t="inlineStr">
+      <c r="C35" s="7" t="inlineStr">
         <is>
           <t>À générer</t>
         </is>
       </c>
-      <c r="D35" s="7" t="inlineStr">
+      <c r="D35" s="6" t="inlineStr">
         <is>
           <t>KAIROS</t>
         </is>
@@ -3275,12 +3293,12 @@
           <t>colosse-de-laile-grise</t>
         </is>
       </c>
-      <c r="C36" s="6" t="inlineStr">
+      <c r="C36" s="7" t="inlineStr">
         <is>
           <t>À générer</t>
         </is>
       </c>
-      <c r="D36" s="7" t="inlineStr">
+      <c r="D36" s="6" t="inlineStr">
         <is>
           <t>KAIROS</t>
         </is>
@@ -3342,12 +3360,12 @@
           <t>brouillage</t>
         </is>
       </c>
-      <c r="C37" s="6" t="inlineStr">
+      <c r="C37" s="7" t="inlineStr">
         <is>
           <t>À générer</t>
         </is>
       </c>
-      <c r="D37" s="7" t="inlineStr">
+      <c r="D37" s="6" t="inlineStr">
         <is>
           <t>KAIROS</t>
         </is>
@@ -3409,12 +3427,12 @@
           <t>extraction-forcee</t>
         </is>
       </c>
-      <c r="C38" s="6" t="inlineStr">
+      <c r="C38" s="7" t="inlineStr">
         <is>
           <t>À générer</t>
         </is>
       </c>
-      <c r="D38" s="7" t="inlineStr">
+      <c r="D38" s="6" t="inlineStr">
         <is>
           <t>KAIROS</t>
         </is>
@@ -3476,12 +3494,12 @@
           <t>pilleuse-depoques</t>
         </is>
       </c>
-      <c r="C39" s="6" t="inlineStr">
+      <c r="C39" s="7" t="inlineStr">
         <is>
           <t>À générer</t>
         </is>
       </c>
-      <c r="D39" s="7" t="inlineStr">
+      <c r="D39" s="6" t="inlineStr">
         <is>
           <t>KAIROS</t>
         </is>
@@ -3543,12 +3561,12 @@
           <t>interrogateur-du-drft</t>
         </is>
       </c>
-      <c r="C40" s="6" t="inlineStr">
+      <c r="C40" s="7" t="inlineStr">
         <is>
           <t>À générer</t>
         </is>
       </c>
-      <c r="D40" s="7" t="inlineStr">
+      <c r="D40" s="6" t="inlineStr">
         <is>
           <t>KAIROS</t>
         </is>
@@ -3610,12 +3628,12 @@
           <t>porteur-cell-codex</t>
         </is>
       </c>
-      <c r="C41" s="6" t="inlineStr">
+      <c r="C41" s="7" t="inlineStr">
         <is>
           <t>À générer</t>
         </is>
       </c>
-      <c r="D41" s="7" t="inlineStr">
+      <c r="D41" s="6" t="inlineStr">
         <is>
           <t>KAIROS</t>
         </is>
@@ -3677,12 +3695,12 @@
           <t>le-moment-opportun</t>
         </is>
       </c>
-      <c r="C42" s="6" t="inlineStr">
+      <c r="C42" s="7" t="inlineStr">
         <is>
           <t>À générer</t>
         </is>
       </c>
-      <c r="D42" s="7" t="inlineStr">
+      <c r="D42" s="6" t="inlineStr">
         <is>
           <t>KAIROS</t>
         </is>
@@ -3749,7 +3767,7 @@
           <t>Forgée</t>
         </is>
       </c>
-      <c r="D43" s="7" t="inlineStr">
+      <c r="D43" s="6" t="inlineStr">
         <is>
           <t>KAIROS</t>
         </is>
@@ -3827,12 +3845,12 @@
           <t>la-comptable</t>
         </is>
       </c>
-      <c r="C44" s="6" t="inlineStr">
+      <c r="C44" s="7" t="inlineStr">
         <is>
           <t>À générer</t>
         </is>
       </c>
-      <c r="D44" s="7" t="inlineStr">
+      <c r="D44" s="6" t="inlineStr">
         <is>
           <t>KAIROS</t>
         </is>
@@ -3899,7 +3917,7 @@
           <t>Forgée</t>
         </is>
       </c>
-      <c r="D45" s="7" t="inlineStr">
+      <c r="D45" s="6" t="inlineStr">
         <is>
           <t>KAIROS</t>
         </is>
@@ -3983,7 +4001,7 @@
           <t>gamin-des-ruelles</t>
         </is>
       </c>
-      <c r="C46" s="6" t="inlineStr">
+      <c r="C46" s="7" t="inlineStr">
         <is>
           <t>À générer</t>
         </is>
@@ -4050,7 +4068,7 @@
           <t>lavandiere-du-fleuve</t>
         </is>
       </c>
-      <c r="C47" s="6" t="inlineStr">
+      <c r="C47" s="7" t="inlineStr">
         <is>
           <t>À générer</t>
         </is>
@@ -4192,7 +4210,7 @@
           <t>macon-du-col</t>
         </is>
       </c>
-      <c r="C49" s="6" t="inlineStr">
+      <c r="C49" s="7" t="inlineStr">
         <is>
           <t>À générer</t>
         </is>
@@ -4259,7 +4277,7 @@
           <t>legionnaire-sans-stele</t>
         </is>
       </c>
-      <c r="C50" s="6" t="inlineStr">
+      <c r="C50" s="7" t="inlineStr">
         <is>
           <t>À générer</t>
         </is>
@@ -4326,7 +4344,7 @@
           <t>baleinier-du-pack</t>
         </is>
       </c>
-      <c r="C51" s="6" t="inlineStr">
+      <c r="C51" s="7" t="inlineStr">
         <is>
           <t>À générer</t>
         </is>
@@ -4393,7 +4411,7 @@
           <t>ours-des-steppes</t>
         </is>
       </c>
-      <c r="C52" s="6" t="inlineStr">
+      <c r="C52" s="7" t="inlineStr">
         <is>
           <t>À générer</t>
         </is>
@@ -4460,7 +4478,7 @@
           <t>poussiere-des-siecles</t>
         </is>
       </c>
-      <c r="C53" s="6" t="inlineStr">
+      <c r="C53" s="7" t="inlineStr">
         <is>
           <t>À générer</t>
         </is>
@@ -4527,7 +4545,7 @@
           <t>temoin-manquant</t>
         </is>
       </c>
-      <c r="C54" s="6" t="inlineStr">
+      <c r="C54" s="7" t="inlineStr">
         <is>
           <t>À générer</t>
         </is>
@@ -4594,7 +4612,7 @@
           <t>messagere-aux-pieds-nus</t>
         </is>
       </c>
-      <c r="C55" s="6" t="inlineStr">
+      <c r="C55" s="7" t="inlineStr">
         <is>
           <t>À générer</t>
         </is>
@@ -4661,7 +4679,7 @@
           <t>griot-sans-archive</t>
         </is>
       </c>
-      <c r="C56" s="6" t="inlineStr">
+      <c r="C56" s="7" t="inlineStr">
         <is>
           <t>À générer</t>
         </is>
@@ -4728,7 +4746,7 @@
           <t>gardienne-du-col</t>
         </is>
       </c>
-      <c r="C57" s="6" t="inlineStr">
+      <c r="C57" s="7" t="inlineStr">
         <is>
           <t>À générer</t>
         </is>
@@ -4795,7 +4813,7 @@
           <t>zone-aveugle</t>
         </is>
       </c>
-      <c r="C58" s="6" t="inlineStr">
+      <c r="C58" s="7" t="inlineStr">
         <is>
           <t>À générer</t>
         </is>
@@ -4862,7 +4880,7 @@
           <t>duelliste-du-pont</t>
         </is>
       </c>
-      <c r="C59" s="6" t="inlineStr">
+      <c r="C59" s="7" t="inlineStr">
         <is>
           <t>À générer</t>
         </is>
@@ -4929,7 +4947,7 @@
           <t>cuirasse-du-detroit</t>
         </is>
       </c>
-      <c r="C60" s="6" t="inlineStr">
+      <c r="C60" s="7" t="inlineStr">
         <is>
           <t>À générer</t>
         </is>
@@ -4996,7 +5014,7 @@
           <t>larchiviste-oublie</t>
         </is>
       </c>
-      <c r="C61" s="6" t="inlineStr">
+      <c r="C61" s="7" t="inlineStr">
         <is>
           <t>À générer</t>
         </is>

</xml_diff>

<commit_message>
feat: Taupe du recrutement (K02) — commune KAIROS 1⚡ 2/1, early agressif
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/SET01-production.xlsx
+++ b/docs/SET01-production.xlsx
@@ -2540,9 +2540,9 @@
           <t>taupe-du-recrutement</t>
         </is>
       </c>
-      <c r="C25" s="7" t="inlineStr">
-        <is>
-          <t>À générer</t>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>Forgée</t>
         </is>
       </c>
       <c r="D25" s="6" t="inlineStr">
@@ -2563,13 +2563,25 @@
       <c r="G25" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H25" s="2" t="inlineStr"/>
-      <c r="I25" s="2" t="inlineStr"/>
-      <c r="J25" s="2" t="inlineStr"/>
+      <c r="H25" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="I25" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>Sans CELL · candidat</t>
+        </is>
+      </c>
       <c r="K25" s="5" t="inlineStr"/>
       <c r="L25" s="2" t="inlineStr"/>
       <c r="M25" s="5" t="inlineStr"/>
-      <c r="N25" s="5" t="inlineStr"/>
+      <c r="N25" s="5" t="inlineStr">
+        <is>
+          <t>Meilleur temps du cycle. Personne ne demande pourquoi.</t>
+        </is>
+      </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
           <t>Non</t>

</xml_diff>

<commit_message>
feat: Exécutant de nuit (K03) — commune KAIROS 2⚡ 2/2, + 1 art alternatif
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/SET01-production.xlsx
+++ b/docs/SET01-production.xlsx
@@ -2619,9 +2619,9 @@
           <t>executant-de-nuit</t>
         </is>
       </c>
-      <c r="C26" s="7" t="inlineStr">
-        <is>
-          <t>À générer</t>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>Forgée</t>
         </is>
       </c>
       <c r="D26" s="6" t="inlineStr">
@@ -2642,13 +2642,25 @@
       <c r="G26" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="H26" s="2" t="inlineStr"/>
-      <c r="I26" s="2" t="inlineStr"/>
-      <c r="J26" s="2" t="inlineStr"/>
+      <c r="H26" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="I26" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>CELL volé · sans registre</t>
+        </is>
+      </c>
       <c r="K26" s="5" t="inlineStr"/>
       <c r="L26" s="2" t="inlineStr"/>
       <c r="M26" s="5" t="inlineStr"/>
-      <c r="N26" s="5" t="inlineStr"/>
+      <c r="N26" s="5" t="inlineStr">
+        <is>
+          <t>Les caméras meurent trente secondes avant son passage. Toujours trente.</t>
+        </is>
+      </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
           <t>Non</t>

</xml_diff>

<commit_message>
feat: Guetteur du moment (K04) — commune KAIROS 3⚡ 2/3, punit les Synchros adverses (2 dégâts au Traveler)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/SET01-production.xlsx
+++ b/docs/SET01-production.xlsx
@@ -2698,9 +2698,9 @@
           <t>guetteur-du-moment</t>
         </is>
       </c>
-      <c r="C27" s="7" t="inlineStr">
-        <is>
-          <t>À générer</t>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>Forgée</t>
         </is>
       </c>
       <c r="D27" s="6" t="inlineStr">
@@ -2721,13 +2721,29 @@
       <c r="G27" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H27" s="2" t="inlineStr"/>
-      <c r="I27" s="2" t="inlineStr"/>
-      <c r="J27" s="2" t="inlineStr"/>
-      <c r="K27" s="5" t="inlineStr"/>
+      <c r="H27" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="I27" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="J27" s="2" t="inlineStr">
+        <is>
+          <t>Sans CELL · observateur</t>
+        </is>
+      </c>
+      <c r="K27" s="5" t="inlineStr">
+        <is>
+          <t>Quand un Traveler adverse active une Synchro, infligez-lui 2 dégâts.</t>
+        </is>
+      </c>
       <c r="L27" s="2" t="inlineStr"/>
       <c r="M27" s="5" t="inlineStr"/>
-      <c r="N27" s="5" t="inlineStr"/>
+      <c r="N27" s="5" t="inlineStr">
+        <is>
+          <t>Il ne regarde pas la ville. Il regarde ce qui s'allume.</t>
+        </is>
+      </c>
       <c r="O27" s="2" t="inlineStr">
         <is>
           <t>Non</t>

</xml_diff>

<commit_message>
feat: Nettoyeuse (K06) — commune KAIROS 4⚡ 3/3, À l'arrivée : 2 dégâts à une unité
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/SET01-production.xlsx
+++ b/docs/SET01-production.xlsx
@@ -2864,9 +2864,9 @@
           <t>nettoyeuse</t>
         </is>
       </c>
-      <c r="C29" s="7" t="inlineStr">
-        <is>
-          <t>À générer</t>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>Forgée</t>
         </is>
       </c>
       <c r="D29" s="6" t="inlineStr">
@@ -2887,13 +2887,29 @@
       <c r="G29" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="H29" s="2" t="inlineStr"/>
-      <c r="I29" s="2" t="inlineStr"/>
-      <c r="J29" s="2" t="inlineStr"/>
-      <c r="K29" s="5" t="inlineStr"/>
+      <c r="H29" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I29" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="J29" s="2" t="inlineStr">
+        <is>
+          <t>Sans CELL · sous-traitance</t>
+        </is>
+      </c>
+      <c r="K29" s="5" t="inlineStr">
+        <is>
+          <t>À l'arrivée : infligez 2 dégâts à une unité.</t>
+        </is>
+      </c>
       <c r="L29" s="2" t="inlineStr"/>
       <c r="M29" s="5" t="inlineStr"/>
-      <c r="N29" s="5" t="inlineStr"/>
+      <c r="N29" s="5" t="inlineStr">
+        <is>
+          <t>La chambre était impeccable. C'est bien le problème.</t>
+        </is>
+      </c>
       <c r="O29" s="2" t="inlineStr">
         <is>
           <t>Non</t>

</xml_diff>